<commit_message>
Update berita 2026-08-05 15:18 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-05.xlsx
+++ b/data/berita_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$457</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$559</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I457"/>
+  <dimension ref="A1:I559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -21913,8 +21913,4802 @@
         </is>
       </c>
     </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Gubernur Sumut kembali berkantor di Nias guna percepat pembangunan</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:02:01 +0700</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Gubernur Sumatera Utara Bobby Nasution kembali berkantor di Kepulauan Nias sebagai wujud berkelanjutan pemerintah ...</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681629/gubernur-sumut-kembali-berkantor-di-nias-guna-percepat-pembangunan</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001032290.jpg</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>11 korban kebakaran KM Mutiara Sentosa II jalani perawatan medis</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:01:34 +0700</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>ANTARA - Dari total 238 korban kebakaran kapal penumpang KM Mutiara Sentosa II yang terevakuasi, sebelas orang di ...</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681625/11-korban-kebakaran-km-mutiara-sentosa-ii-jalani-perawatan-medis</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_11-KORBAN-KEBAKARAN-KM-MUTIARA-SENTOSA-II-JALANI-PERAWATAN-MEDIS.jpg</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Pemkot Solo siapkan kios bagi pedagang terdampak tutupnya PGS</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:01:32 +0700</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Solo menyiapkan kios dan los di sejumlah pasar tradisional bagi pedagang yang terdampak ...</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681600/pemkot-solo-siapkan-kios-bagi-pedagang-terdampak-tutupnya-pgs</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PEMKOT-SOLO-SIAPKAN-KIOS-BAGI-PEDAGANG-TERDAMPAK-TUTUPNYA-PGS.jpg</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Akademisi: Perlu ada sosialisasi dan evaluasi atas penerapan UU TPKS</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:00:39 +0700</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Akademisi dari Fakultas Hukum Universitas Katolik Parahyangan (Unpar) mengatakan perlu adanya sosialisasi dan evaluasi ...</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681627/akademisi-perlu-ada-sosialisasi-dan-evaluasi-atas-penerapan-uu-tpks</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000012935.jpg</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>KSP jelaskan alasan KDMP dibangun di kaki gunung Ciremai</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:56:56 +0700</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>ANTARA - Kepala Staf Kepresidenan Dudung Abdurachman menyebut kehadiran Koperasi Desa Merah Putih atau KDMP di ...</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681552/ksp-jelaskan-alasan-kdmp-dibangun-di-kaki-gunung-ciremai</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-205638_1.jpg</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Indonesia jajaki peluang penempatan pekerja migran ke Slowakia</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:56:17 +0700</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Kementerian Pelindungan Pekerja Migran Indonesia (P2MI) menjajaki peluang perluasan penempatan pekerja migran Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681624/indonesia-jajaki-peluang-penempatan-pekerja-migran-ke-slowakia</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/405.jpg</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>SIG bidik penguatan pasar di Jawa Barat lewat Semen Kujang</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:53:49 +0700</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>PT Semen Indonesia (Persero) Tbk (SIG) memperkuat upaya dominasi pasar di Jawa Barat dengan menghadirkan kembali Semen ...</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681620/sig-bidik-penguatan-pasar-di-jawa-barat-lewat-semen-kujang</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-20.35.21.jpeg</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>KPK duga pejabat Kemenhut dapat 12.500 dolar Singapura dari Suhardiman</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:52:29 +0700</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi menduga pejabat di Kementerian Kehutanan mendapatkan penerimaan uang sebesar 12.500 dolar ...</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681619/kpk-duga-pejabat-kemenhut-dapat-12500-dolar-singapura-dari-suhardiman</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7411.jpg</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>42 persen tiket terjual, MotoGP Indonesia 2026 dikemas lebih menarik</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:50:44 +0700</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>ANTARA - Penjualan tiket ajang balap motor bergengsi dunia, MotoGP seri Indonesia tahun 2026, mencatatkan ...</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681607/42-persen-tiket-terjual-motogp-indonesia-2026-dikemas-lebih-menarik</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_42-PERSEN-TIKET-TERJUAL-MOTOGP-INDONESIA-2026-DIKEMAS-LEBIH-MENARIK_1.jpg</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Pemprov DKI terima aset fasos-fasum senilai Rp2,27 triliun</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:47:56 +0700</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta menerima aset fasilitas sosial dan fasilitas umum (fasos/fasum) dari para ...</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681616/pemprov-dki-terima-aset-fasos-fasum-senilai-rp227-triliun</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000315242.jpg</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Kenapa pikiran selalu aktif saat mau tidur? Ini penyebab dan cara mengatasinya</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:47:44 +0700</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Tubuh sudah terasa lelah, mata mulai mengantuk, tetapi begitu berbaring di tempat tidur, pikiran justru semakin aktif. ...</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681613/kenapa-pikiran-selalu-aktif-saat-mau-tidur-ini-penyebab-dan-cara-mengatasinya</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/15/banun.jpg</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Otto: Sistem kekayaan intelektual ideal beri manfaat sosial-ekonomi</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:47:14 +0700</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Koordinator Bidang Hukum, Hak Asasi Manusia, Imigrasi, dan Pemasyarakatan Otto Hasibuan mengatakan sistem ...</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681609/otto-sistem-kekayaan-intelektual-ideal-beri-manfaat-sosial-ekonomi</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000471686.jpg</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Pramono setuju modifikasi cuaca dilakukan dua kali sepekan</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:44:21 +0700</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta, Pramono Anung memberikan persetujuan untuk dilakukan operasi modifikasi cuaca (OMC) setiap satu ...</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681604/pramono-setuju-modifikasi-cuaca-dilakukan-dua-kali-sepekan</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000315232_1.jpg</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Pemkab Aceh Besar salurkan air bersih ke warga terdampak kekeringan</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:43:48 +0700</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>ANTARA - Kemarau yang melanda kabupaten Aceh Besar dalam beberapa pekan terakhir, menyebabkan pasokan air bersih ...</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681487/pemkab-aceh-besar-salurkan-air-bersih-ke-warga-terdampak-kekeringan</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PEMKAB-ACEH-BESAR-SALURKAN-AIR-BERSIH-KE-WARGA-TERDAMPAK-KEKERINGAN.jpg</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Pembangunan MRT, Dishub DKI rekayasa lalin di kawasan Stasiun Kota</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:40:21 +0700</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Dinas Perhubungan (Dishub) DKI Jakarta menerapkan rekayasa lalu lintas di kawasan Stasiun Glodok dan Stasiun Kota ...</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681596/pembangunan-mrt-dishub-dki-rekayasa-lalin-di-kawasan-stasiun-kota</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/20/revitalisasi-stasiun-mrt-bundaran-hi-2775419.jpg</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Dudung: Koordinasi lintas sektor kunci penyelesaian program prioritas</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:40:18 +0700</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Kepala Staf Kepresidenan Jenderal TNI (Purn.) Dudung Abdurachman mengatakan koordinasi lintas sektor yang difasilitasi ...</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681595/dudung-koordinasi-lintas-sektor-kunci-penyelesaian-program-prioritas</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/482452.jpg</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Menkeu Purbaya tak setuju gaji manajer KDKMP sebesar Rp16,25 juta</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:40:08 +0700</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>ANTARA - Beredar informasi di media sosial yang menyebut gaji manajer koperasi desa kelurahan merah putih (KDKMP) ...</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681512/menkeu-purbaya-tak-setuju-gaji-manajer-kdkmp-sebesar-rp1625-juta</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_MENKEU-PURBAYA-TAK-SETUJU-GAJI-MANAJER-KDKMP-SEBESAR-RP16-25-JUTA.jpg</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Apa Itu sleep hygiene? Ini manfaat dan 10 cara menerapkannya agar tidur nyenyak</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:37:14 +0700</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Banyak orang mengira sulit tidur hanya disebabkan oleh stres atau terlalu banyak minum kopi. Padahal, kualitas tidur ...</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681593/apa-itu-sleep-hygiene-ini-manfaat-dan-10-cara-menerapkannya-agar-tidur-nyenyak</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/10/tidur.jpg</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Apple menduga banyak mantan karyawan bocorkan data rahasia ke OpenAI</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:36:39 +0700</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Apple menyatakan banyak mantan karyawannya diduga mengambil informasi rahasia perusahaan sebelum bergabung dengan ...</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681592/apple-menduga-banyak-mantan-karyawan-bocorkan-data-rahasia-ke-openai</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/thumbs_b_c_c48eb58d9c1e7c83fd91f3633ecd20ec.jpg</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Dubes Pakistan: RI punya peran penting dorong resolusi Kashmir</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:36:35 +0700</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Duta Besar Pakistan untuk Indonesia, Zahid Hafeez Chaudhri, menilai bahwa Indonesia memiliki peran penting bersama ...</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681589/dubes-pakistan-ri-punya-peran-penting-dorong-resolusi-kashmir</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000010449.jpg</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>KPK sebut saksi kasus KPP Banjarmasin kembalikan uang 530.000 dolar AS</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:36:15 +0700</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi menyatakan salah satu saksi dalam pengembangan kasus dugaan korupsi yang menjerat ...</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681585/kpk-sebut-saksi-kasus-kpp-banjarmasin-kembalikan-uang-530000-dolar-as</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/27/pemeriksaan-tersangka-kasus-korupsi-restitusi-pajak-2739814.jpg</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>KPK duga Menhut belum kembalikan seluruh uang Suhardiman Amby</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:33:20 +0700</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi menduga Menteri Kehutanan Raja Juli Antoni belum mengembalikan seluruh uang dalam amplop ...</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681581/kpk-duga-menhut-belum-kembalikan-seluruh-uang-suhardiman-amby</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/0e9984fc-378c-48cd-96a2-13ba508fcc3e.jpeg</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Menkum harap Rencana Induk KI Nasional 2027–2036 jadi PSN</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:33:15 +0700</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Menteri Hukum (Menkum) Supratman Andi Agtas mengharapkan Rencana Induk Kekayaan Intelektual (KI) Nasional ...</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681577/menkum-harap-rencana-induk-ki-nasional-2027-2036-jadi-psn</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000471680.jpg</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Sudinsos Jaksel distribusi 690 alat bantu fisik bagi warga yang butuh</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:31:31 +0700</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Suku Dinas Sosial Jakarta Selatan telah mendistribusikan sebanyak 690 alat bantu fisik kepada warga yang membutuhkan ...</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681576/sudinsos-jaksel-distribusi-690-alat-bantu-fisik-bagi-warga-yang-butuh</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001013673.jpg</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>ASDP perkuat transformasi operasional lewat standar baru keselamatan</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:30:37 +0700</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>PT ASDP Indonesia Ferry (Persero) mengimplementasikan standar baru keselamatan melalui program sterilisasi pelabuhan ...</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681573/asdp-perkuat-transformasi-operasional-lewat-standar-baru-keselamatan</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-18.08.02.jpeg</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>7 cara mempersiapkan anak sambut kelahiran adik agar tidak cemburu</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:30:18 +0700</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Kehadiran anggota keluarga baru dapat menjadi momen bahagia sekaligus tantangan bagi anak pertama. Persiapan sejak dini ...</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681571/7-cara-mempersiapkan-anak-sambut-kelahiran-adik-agar-tidak-cemburu</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/15/pexels-migs-reyes-4205505.jpg</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Jumlah penduduk miskin di Jakarta 432 ribu orang pada Maret 2026</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:29:25 +0700</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Badan Pusat Statistik (BPS) DKI Jakarta mengemukakan jumlah penduduk miskin di Jakarta sebanyak 432,62 ribu orang pada ...</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681568/jumlah-penduduk-miskin-di-jakarta-432-ribu-orang-pada-maret-2026</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000315200.jpg</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>KKP manfaatkan TKD untuk budi daya ikan tematik di DIY</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:24:44 +0700</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Kelautan dan Perikanan (KKP) akan meluncurkan Program Budi Daya Perikanan Tematik di 64 kalurahan ...</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681401/kkp-manfaatkan-tkd-untuk-budi-daya-ikan-tematik-di-diy</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-194302.jpg</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Sudinsos Jaksel jangkau 644 PPKS hingga Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:23:22 +0700</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Suku Dinas Sosial Jakarta Selatan mencatat telah menjangkau 644 Pemerlu Pelayanan Kesejahteraan Sosial (PPKS) sepanjang ...</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681565/sudinsos-jaksel-jangkau-644-ppks-hingga-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001013669.jpg</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Posisi tidur yang baik untuk kesehatan, mana yang paling dianjurkan?</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:21:18 +0700</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Tidur merupakan waktu bagi tubuh untuk memulihkan energi dan memperbaiki berbagai fungsi penting. Namun, selain durasi ...</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681564/posisi-tidur-yang-baik-untuk-kesehatan-mana-yang-paling-dianjurkan</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/28/atur.jpg</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Argentina sesalkan Brasil menurunkan tingkat hubungan diplomatik</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:21:06 +0700</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Argentina pada Selasa (4/8) menyatakan penyesalannya atas keputusan Brasil yang menurunkan hubungan diplomatik ...</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681563/argentina-sesalkan-brasil-menurunkan-tingkat-hubungan-diplomatik</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000023_20260805_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Menbud nilai perancang busana mampu promosikan wastra Indonesia</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:19:55 +0700</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Menteri Kebudayaan Fadli Zon menilai perancang busana mampu mempromosikan wastra Indonesia, termasuk batik, kepada ...</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681561/menbud-nilai-perancang-busana-mampu-promosikan-wastra-indonesia</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-04-at-05.45.36.jpeg</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>PN gelar sidang praperadilan Febrie Adriansyah pada 18-19 Agustus</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:19:35 +0700</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Pengadilan Negeri (PN) Jakarta Selatan menjadwalkan sidang perdana dua gugatan praperadilan yang diajukan mantan Jaksa ...</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681557/pn-gelar-sidang-praperadilan-febrie-adriansyah-pada-18-19-agustus</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001013665.jpg</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Polres Cilegon siapkan kantong parkir tertibkan truk tambang</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:19:03 +0700</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>ANTARA - Polres Cilegon menyiapkan kantong parkir untuk menampung truk angkutan tambang yang melanggar jam operasional ...</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681476/polres-cilegon-siapkan-kantong-parkir-tertibkan-truk-tambang</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-203312.jpg</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Pemprov Jabar ubah skema layanan BRT hemat anggaran Rp10 miliar</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:16:11 +0700</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Jawa Barat mengubah skema pengelolaan layanan Bus Rapid Transit (BRT) Metro Jabar Trans ...</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681535/pemprov-jabar-ubah-skema-layanan-brt-hemat-anggaran-rp10-miliar</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_PEMPROV-JABAR-UBAH-SKEMA-LAYANAN-BRT-HEMAT-ANGGARAN-RP10-MILIAR.jpg</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Menteri PPPA tekankan pentingnya pesantren ramah santri</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:16:00 +0700</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Pemberdayaan Perempuan dan Perlindungan Anak (PPPA) Arifatul Choiri Fauzi di Malang, Jawa Timur, Rabu ...</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681448/menteri-pppa-tekankan-pentingnya-pesantren-ramah-santri</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-201229.jpg</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Wamendagri minta daerah bangun ekosistem Koperasi Merah Putih</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:14:37 +0700</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Dalam Negeri (Wamendagri) Bima Arya Sugiarto meminta kepala daerah membangun ekosistem Koperasi ...</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681548/wamendagri-minta-daerah-bangun-ekosistem-koperasi-merah-putih</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000580528.jpg</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Job Fair Kabupaten Bogor sediakan 6.056 lowongan kerja</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:13:55 +0700</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kabupaten Bogor menggelar Job Fair Kabupaten Bogor 2026 dengan menyediakan 6.056 lowongan kerja ...</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681523/job-fair-kabupaten-bogor-sediakan-6056-lowongan-kerja</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_JOB-FAIR-KABUPATEN-BOGOR-SEDIAKAN-6.056-LOWONGAN-KERJA.jpg</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Balsa Sekulic bertekad membawa Persib juara Piala Presiden 2026</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:13:21 +0700</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Striker Persib Bandung Balsa Sekulic bertekad membawa timnya menjuarai Piala Presiden 2026 meski harus menghadapi ...</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681547/balsa-sekulic-bertekad-membawa-persib-juara-piala-presiden-2026</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG-20260805-WA0008_2.jpg</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya gagalkan peredaran empat kilogram ganja di Jakbar</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:13:06 +0700</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Direktorat Reserse Narkoba Polda Metro Jaya kembali berhasil menggagalkan peredaran narkotika jenis ganja seberat ...</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681543/polda-metro-jaya-gagalkan-peredaran-empat-kilogram-ganja-di-jakbar</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_20260805_203415.v1.jpg</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Electronic Arts resmi diakuisisi Arab Saudi senilai Rp982 triliun</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:12:25 +0700</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Perusahaan gim Electronic Arts (EA) yang dikenal sebagai pencipta gim EA FC dan The Sims resmi menjadi perusahaan ...</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681540/electronic-arts-resmi-diakuisisi-arab-saudi-senilai-rp982-triliun</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000141394.jpg</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Mendagri: perbaikan fasum Padang akibat banjir gunakan dana presiden</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:12:06 +0700</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Dalam Negeri Tito Karnavian mengusulkan agar pemerintah daerah dapat memanfaatkan dana tambahan ...</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681492/mendagri-perbaikan-fasum-padang-akibat-banjir-gunakan-dana-presiden</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-204650.jpg</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Menteri PPPA: Nilai agama hingga etika lindungi tumbuh kembang anak</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:11:50 +0700</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Menteri Pemberdayaan Perempuan dan Perlindungan Anak (PPPA) Arifah Fauzi menyatakan penanaman nilai agama, budi ...</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681539/menteri-pppa-nilai-agama-hingga-etika-lindungi-tumbuh-kembang-anak</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001400813.jpg</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Bendera raksasa dikibarkan, Bogor gaungkan semangat nasionalisme</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:10:33 +0700</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>ANTARA - Menjelang HUT ke-81 Kemerdekaan RI, Pemerintah Kabupaten Bogor mengibarkan bendera Merah Putih berukuran 30 x ...</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681461/bendera-raksasa-dikibarkan-bogor-gaungkan-semangat-nasionalisme</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-202347.jpg</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>KPK sita 150.000 dolar AS terkait pengembangan kasus KPP Banjarmasin</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:09:57 +0700</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi menyita uang tunai senilai 150.000 dolar AS dari penggeledahan di dua lokasi terkait ...</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681532/kpk-sita-150000-dolar-as-terkait-pengembangan-kasus-kpp-banjarmasin</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/15/pemeriksaan-tersangka-dian-jaya-demega-2772685.jpg</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Sudinhub Jakut tindak puluhan motor yang parkir liar di Sunter Agung</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:07:59 +0700</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Suku Dinas Perhubungan (Sudinhub) Jakarta Utara menindak tegas puluhan motor yang kedapatan parkir secara liar di ...</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681528/sudinhub-jakut-tindak-puluhan-motor-yang-parkir-liar-di-sunter-agung</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-20.26.54.jpeg</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Persebaya tak gentar hadapi Persib di final Piala Presiden 2026</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:07:38 +0700</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Pemain Persebaya Surabaya Francisco Rivera mengungkapkan timnya sudah siap menghadapi Persib Bandung pada final Piala ...</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681524/persebaya-tak-gentar-hadapi-persib-di-final-piala-presiden-2026</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG-20260805-WA0005.jpg</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Pemkab Bangka Barat perkuat ekonomi desa melalui Sekolah BUMDesa</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:06:16 +0700</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten (Pemkab) Bangka Barat, Provinsi Kepulauan Bangka Belitung (Babel), berupaya memperkuat ekonomi ...</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681520/pemkab-bangka-barat-perkuat-ekonomi-desa-melalui-sekolah-bumdesa</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_20260805_162408.jpg</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Satgas PRR minta 16 K/L segera eksekusi program rehab-rekon</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:04:30 +0700</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Menteri Dalam Negeri Muhammad Tito Karnavian selaku Ketua Satuan Tugas Percepatan Rehabilitasi dan Rekonstruksi ...</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681515/satgas-prr-minta-16-k-l-segera-eksekusi-program-rehab-rekon</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000580507.jpg</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Jumlah pengangguran di Jakarta turun 10 ribu orang pada Mei 2026</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:01:27 +0700</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Badan Pusat Statistik (BPS) DKI Jakarta mencatat jumlah pengangguran di ibu kota mengalami penurunan 10 ribu orang pada ...</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681509/jumlah-pengangguran-di-jakarta-turun-10-ribu-orang-pada-mei-2026</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000315189.jpg</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>200 museum dan cagar budaya akan direvitalisasi, langkah Sumut diapresiasi</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:58:58 +0700</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Menteri Kebudayaan Fadli Zon mengatakan bahwa pada tahun ini pihaknya akan merevitalisasi hampir 200 museum dan ...</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681500/200-museum-dan-cagar-budaya-akan-direvitalisasi-langkah-sumut-diapresiasi</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/18/penunjukan-pelaksana-tugas-pengelolaan-keraton-kasunanan-solo-2707786.jpg</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>KSP pastikan kesiapan operasional Sekolah Rakyat Terintegrasi Bandung</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:19:29 +0700</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Kantor Staf Presiden (KSP) melakukan verifikasi lapangan guna memastikan kesiapan operasional Sekolah Rakyat ...</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681449/ksp-pastikan-kesiapan-operasional-sekolah-rakyat-terintegrasi-bandung</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_0966.jpg</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>BP BUMN-Kemenkeu bahas relaksasi perpajakan untuk transformasi BUMN</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:06:16 +0700</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Kepala Badan Pengaturan (BP) BUMN sekaligus COO Danantara Dony Oskaria bertemu Menteri Keuangan Purbaya Yudhi ...</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681429/bp-bumn-kemenkeu-bahas-relaksasi-perpajakan-untuk-transformasi-bumn</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/COO-Danantara-temui-Menteri-Keuangan-050826-Bay-1.jpg</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Staf RSUD di Tasik Terancam Disanksi Gegara Ikut Nyinyir ke Pasien BPJS</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:05:04 +0700</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Faizal Amiruddin</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Seorang pegawai RSUD dr Soekardjo Tasikmalaya terancam sanksi setelah berkomentar kasar tentang pasien BPJS. Pihak rumah sakit sedang menindaklanjuti kasus ini.</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606160/staf-rsud-di-tasik-terancam-disanksi-gegara-ikut-nyinyir-ke-pasien-bpjs</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/11/rsud-dr-soekardjo-tasikmalaya-1781150055801_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Gempa M 5,3 Terjadi di Pangandaran</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:03:43 +0700</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Gempa bumi dengan magnitudo (M) 5,3 terjadi di Pangandaran, Jawa Barat. Gempa ada pada kedalaman 18 kilometer.</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606157/gempa-m-5-3-terjadi-di-pangandaran</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/08/ilustrasi-gempa-1780909642348_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Belasan Pekerja Dapur MBG di Bima Diduga Terpapar Hepatitis</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:02:21 +0700</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Rafiin</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Belasan relawan dapur Makan Bergizi Gratis di Bima diduga terinfeksi hepatitis. Puskesmas menemukan 15 orang reaktif setelah skrining kesehatan.</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606155/belasan-pekerja-dapur-mbg-di-bima-diduga-terpapar-hepatitis</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/27/32-ribu-pegawai-inti-mbg-bakal-diangkat-jadi-asn-pppk-1769488598657_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Ekspedisi Merah Putih Hadirkan Nasionalisme, Cinta Alam &amp;amp; Ceria di Ujung Siak</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:59:48 +0700</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Tim Ekspedisi Merah Putih Polda Riau jangkau Kampung Teluk Lanus, menanam 1.000 mangrove, dan memberikan bansos serta peralatan sekolah untuk masyarakat.</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606152/ekspedisi-merah-putih-hadirkan-nasionalisme-cinta-alam-ceria-di-ujung-siak</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/ekspedisi-merah-putih-jangkau-ujung-siak-menanam-1000-mangrove-dan-menyerahkan-bansos-kepada-masyarakat-1785941846802_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Ekspedisi Merah Putih Hadirkan Nasionalisme, Cinta Alam &amp;amp; Ceria di Ujung Siak</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:59:48 +0700</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Tim Ekspedisi Merah Putih Polda Riau menanam 1.000 mangrove, menyerahkan bansos di Kampung Teluk Lanus, meningkatkan semangat nasionalisme dan cinta alam.</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/melindungi-tuah-marwah/d-8606159/ekspedisi-merah-putih-hadirkan-nasionalisme-cinta-alam-ceria-di-ujung-siak</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/ekspedisi-merah-putih-jangkau-ujung-siak-menanam-1000-mangrove-dan-menyerahkan-bansos-kepada-masyarakat-1785941846802_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Kemensos Tangguhkan 1,49 Juta Penerima Bansos Terindikasi Judi Online</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:46:55 +0700</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Kemensos tangguhkan 1.494.652 Keluarga Penerima Manfaat Program Sembako yang terindikasi judi online. Proses verifikasi dilakukan untuk memastikan kelayakan.</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606144/kemensos-tangguhkan-1-49-juta-penerima-bansos-terindikasi-judi-online</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/kemensos-tangguhkan-149-juta-penerima-bansos-terindikasi-judi-online-1785941114903_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>BPS Sebut Jumlah Orang Terserap Pasar Kerja Meningkat di Mei 2026</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:45:43 +0700</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>BPS melaporkan jumlah penduduk bekerja Mei 2026 mencapai 148,19 juta, meningkat 522 ribu. Sektor Akomodasi dan Makan Minum jadi penyerap tenaga kerja terbanyak.</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606075/bps-sebut-jumlah-orang-terserap-pasar-kerja-meningkat-di-mei-2026</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/05/kepala-bps-amalia-adininggar-widyasanti-1777954089390_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Mahasiswi PPDS Diduga Hina Pasien BPJS 'Orang Have', UGM Turun Tangan</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:43:00 +0700</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Serly Putri Jumbadi</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Viral komentar nyinyir mahasiswi UGM, Elda Putri, terkait pasien BPJS Kesehan. UGM investigasi dan sanksi akan dijatuhkan jika terbukti bersalah.</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606140/mahasiswi-ppds-diduga-hina-pasien-bpjs-orang-have-ugm-turun-tangan</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/01/15/ilustrasi-kamar-rumah-sakit_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap 3 Anggota Ormas Hendak Rebut Ruko Warga di Surabaya</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:25:37 +0700</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Aprilia Devi</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Polisi amankan tiga anggota ormas terkait penyerobotan ruko di Surabaya. Sementara pelaku lain masih diburu.</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606131/polisi-tangkap-3-anggota-ormas-hendak-rebut-ruko-warga-di-surabaya</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/07/25/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Waka MPR Ungkap Pentingnya Kolaborasi Pengelolaan Warisan Budaya</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:16:43 +0700</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Hana Nushratu Uzma</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR Lestari Moerdijat menekankan pentingnya pelestarian warisan budaya. Kolaborasi pemerintah dan masyarakat penting dalam menjaga aset budaya.</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606119/waka-mpr-ungkap-pentingnya-kolaborasi-pengelolaan-warisan-budaya</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/03/03/lestari-moerdijat.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Hujan Buatan Jadi Harapan Saat Kemarau Berkepanjangan</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:13:26 +0700</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Haris Fadhil</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Kemarau telah memicu kekeringan di berbagai daerah di Indonesia. Kini, hujan buatan menjadi salah satu harapan untuk mengatasi kekeringan.</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606115/hujan-buatan-jadi-harapan-saat-kemarau-berkepanjangan</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/01/kemarau-ancam-ribuan-hektare-sawah-di-bekasi-kekeringan-berpotensi-meluas-1785576721983_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Kembangkan Kewirausahaan, Gubernur Sumsel Gagas Kampus Sekolah Ekspor</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:09:45 +0700</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Gubernur Sumsel luncurkan Kampus Sekolah Ekspor, kampus outdoor pertama di Indonesia, untuk dorong kewirausahaan dan pengusaha muda berorientasi ekspor.</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606103/kembangkan-kewirausahaan-gubernur-sumsel-gagas-kampus-sekolah-ekspor</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/kembangkan-kewirausahaan-gubernur-sumsel-gagas-kampus-sekolah-ekspor-1785938837794_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>DLH Bogor Identifikasi Perusahaan Diduga Bikin Air Kali Bekasi Hitam Bak Oli</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:04:36 +0700</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Muchamad Sholihin</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Dinas LH Kabupaten Bogor uji laboratorium dan susur sungai terkait pencemaran air hitam di Sungai Cileungsi. Perusahaan terancam sanksi jika terbukti bersalah.</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606093/dlh-bogor-identifikasi-perusahaan-diduga-bikin-air-kali-bekasi-hitam-bak-oli</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/video-air-kali-bekasi-berwarna-hitam-mirip-oli-bekas-viral-di-media-sosial-medsos-kualitas-air-tersebut-menurun-karena-ada-dug-1785929406139_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Pemerintah Bakal Tindak Lanjuti Dugaan Keracunan Makanan di Jayapura</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:02:21 +0700</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulias</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Wamendagri Ribka Haluk menegaskan perhatian pemerintah terhadap dugaan keracunan makanan di Jayapura. Tim akan turun untuk verifikasi dan evaluasi situasi.</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606089/pemerintah-bakal-tindak-lanjuti-dugaan-keracunan-makanan-di-jayapura</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/wakil-menteri-dalam-negeri-wamendagri-ribka-haluk-1785938501104.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Israel Gempur Lebanon Selatan, Tuduh Hizbullah Langgar Gencatan Senjata</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:01:12 +0700</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Militer Israel menyerang target di Lebanon selatan, menuduh Hizbullah melanggar gencatan senjata. Warga diminta mengungsi.</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606087/israel-gempur-lebanon-selatan-tuduh-hizbullah-langgar-gencatan-senjata</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/lebanon-israel-iran-us-war-1785938380565_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Latihan Gabungan TNI 2026 Peragakan Kemampuan Tempur Tiga Matra</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:56:06 +0700</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Grandyos Zafna</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>TNI menggelar Operasi Terintegrasi 2026 di Kepulauan Riau dengan simulasi tempur tiga matra yang melibatkan rudal, drone, dan pasukan marinir.</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/foto-news/d-8605344/latihan-gabungan-tni-2026-peragakan-kemampuan-tempur-tiga-matra</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/latihan-operasi-tni-terintegrasi-2026-1785913841495.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>KPK Geledah 2 Rumah Kasus Suap Pajak Banjarmasin, Amankan USD 150 Ribu</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:54:12 +0700</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>KPK menggeledah Kantor Pajak Pratama Banjarmasin, Bandung, dan Tangerang, menyita total USD 150 ribu terkait kasus korupsi restitusi pajak.</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606077/kpk-geledah-2-rumah-kasus-suap-pajak-banjarmasin-amankan-usd-150-ribu</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/12/jubir-kpk-budi-prasetyo-1778596449122_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Viral Anak Curhat Ibunya Meninggal Usai Ditolak Masuk IGD RS di Lampung</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:40:08 +0700</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Tommy Saputra</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Viral curhatan anak tentang ibunya yang diduga ditolak di IGD RSUDAM Lampung, kini ibu tersebut meninggal. RSUDAM bantah penolakan dan akan lakukan evaluasi.</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606065/viral-anak-curhat-ibunya-meninggal-usai-ditolak-masuk-igd-rs-di-lampung</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/10/11/ilustrasi-rumah-sakit_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>10 Hari Dirawat di RS, Istri Korban Pembunuhan Sekeluarga di Palu Meninggal</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:39:12 +0700</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Rangga Musabar</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Nurhanisa, istri Jamil yang menjadi korban pembunuhan di Palu, meninggal setelah 10 hari perawatan.</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606063/10-hari-dirawat-di-rs-istri-korban-pembunuhan-sekeluarga-di-palu-meninggal</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/pembunuhan-satu-keluarga-di-jalan-pdam-kelurahan-duyu-kecamatan-tatanga-kota-palu-1785135255984_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>BPS RI &amp;amp; MOSPI India Tandatangani Kerja Sama untuk Penguatan Statistik</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:37:07 +0700</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Hana Nushratu</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Kepala BPS RI Amalia Adininggar menghadiri pertemuan NSO BRICS di India, menandatangani LOI dengan India untuk kolaborasi statistik dan pengembangan digital.</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606061/bps-ri-mospi-india-tandatangani-kerja-sama-untuk-penguatan-statistik</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/bps-ri-mospi-india-tandatangani-kerja-sama-untuk-penguatan-statistik-1785936933919_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Mendagri Minta Walkot Pakai Rp 200 M Perbaiki Saluran Air Imbas Banjir Padang</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:36:07 +0700</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Mendagri Tito memastikan penanganan banjir di Kota Padang. Dia juga meminta Wali Kota Padang memanfaatkan anggaran untuk membenahi infrastruktur imbas banjir.</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606058/mendagri-minta-walkot-pakai-rp-200-m-perbaiki-saluran-air-imbas-banjir-padang</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/mendagri-tito-karnavian-eva-safitridetikcom-1785920328767_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Program JKN Jadi Penopang Harapan Herna di Balik Rutinitas Cuci Darah</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:30:42 +0700</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Hana Nushratu</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Herna Sumiratna, pasien hemodialisis, bersyukur atas dukungan Program JKN yang jamin biaya pengobatan. Ia berharap program ini terus berlanjut untuk masyarakat.</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606051/program-jkn-jadi-penopang-harapan-herna-di-balik-rutinitas-cuci-darah</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/jkn-menjadi-penopang-harapan-herna-di-balik-rutinitas-cuci-darah-1785936544109_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Yang Diketahui soal Rencana AS Tutup Konsulat di Medan</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:13:07 +0700</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>AS akan menutup lima misi diplomatik asing, termasuk Konsulat Jenderal AS di Medan, Indonesia. Kebijakan ini menjadi hal yang jarang terjadi. Apa alasannya?</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606027/yang-diketahui-soal-rencana-as-tutup-konsulat-di-medan</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/01/19/ribuan-bendera-as-meriahkan-pelantikan-joe-biden-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Menko Polkam Minta TNI-Polri Tingkatkan Patroli Cegah Warga Main Hakim Sendiri</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:11:01 +0700</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Rumondang Naibaho</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Menko Polkam Djamari Chaniago menyoroti aksi warga main hakim sendiri. Ia minta peningkatan patroli TNI-Polri untuk pencegahan konflik.</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606024/menko-polkam-minta-tni-polri-tingkatkan-patroli-cegah-warga-main-hakim-sendiri</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/menko-polkam-pastikan-situasi-nasional-terkendali-minta-masyarakat-tak-terpengaruh-hoaks-1785916804844_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>136 Siswa hingga Kepala Sekolah SMPN 5 Rembang Alami Diare Massal</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:10:31 +0700</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Mukhammad Fadlil</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Sebanyak 136 siswa di SMP Negeri 5 Rembang dilaporkan mengalami diare. Sejumlah guru dan tenaga tata usaha (TU) juga mengalami keluhan serupa.</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606023/136-siswa-hingga-kepala-sekolah-smpn-5-rembang-alami-diare-massal</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/keracunan-mbg-1785927316244_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Saksi Kasus Suap Eks Kepala Kantor Pajak Banjarmasin Kembalikan Duit Rp 9,5 M</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:47:30 +0700</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>KPK periksa saksi dalam kasus korupsi pajak di Banjarmasin. Saksi kembalikan uang Rp 9,5 miliar.</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8605991/saksi-kasus-suap-eks-kepala-kantor-pajak-banjarmasin-kembalikan-duit-rp-9-5-m</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/03/02/gedung-baru-kpk-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Wamendagri Minta Pemda Papua Pastikan Penyaluran Dana Otsus Tepat Waktu</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:45:26 +0700</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Wamendagri Ribka Haluk mendorong pemerintah daerah di Papua untuk segera menyelesaikan penyaluran Dana Otsus Tahap II 2026 secara akuntabel dan tepat waktu.</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8605970/wamendagri-minta-pemda-papua-pastikan-penyaluran-dana-otsus-tepat-waktu</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/wamendagri-minta-pemda-papua-pastikan-penyaluran-dana-otsus-tepat-waktu-1785932810840_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Dukung Industri Kecantikan RI, IndoBeauty Expo 2026 Resmi Dibuka</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:42:15 +0700</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>IndoBeauty Expo 2026 resmi dibuka, menjadi platform strategis bagi industri kecantikan. Pameran ini mendorong inovasi, kolaborasi, dan peluang bisnis global.</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606045/dukung-industri-kecantikan-ri-indobeauty-expo-2026-resmi-dibuka</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/07/indobeauty-expo-2025-1754548154322.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Wanita Dilecehkan di KRL Tujuan Depok, KCI Akan Tindak Pelanggar</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:38:11 +0700</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Seorang wanita diduga menjadi korban pelecehan seksual di dalam KRL rute Jakarta Kota-Depok oleh seorang pria. KCI akan menindak pelaku pelecehan.</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8605985/wanita-dilecehkan-di-krl-tujuan-depok-kci-akan-tindak-pelanggar</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/30/ilustrasi-kereta-rel-listrik-krl-dok-kci_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Korlantas Polri Catat Korban Tewas Laka Lantas Semester I Turun 22,92 Persen</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:31:00 +0700</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Herianto Batubara</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Satu bulan sejak kepemimpinan Kakorlantas Polri Irjen Wibowo, kinerja keselamatan lalu lintas menunjukkan tren positif.</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8605979/korlantas-polri-catat-korban-tewas-laka-lantas-semester-i-turun-22-92-persen</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/kakorlantas-polri-irjen-wibowo-1785932835877_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>DPD Undang JK Hadiri Sidang Tahunan: Kumpulkan Tokoh Bangsa</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:45:24 +0700</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Ketua DPD Sultan Najamudin mengundang Jusuf Kalla untuk hadir dalam Sidang Tahunan MPR pada 14 Agustus, menyambut HUT RI ke-81.</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8605927/dpd-undang-jk-hadiri-sidang-tahunan-kumpulkan-tokoh-bangsa</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/ketua-dpd-memberikan-undangan-sidang-tahunan-mpr-ke-jk-1785930226552_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Dapur MBG Wajib Urus SLHS Paling Lambat 10 Agustus atau Tutup Permanen!</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:24:13 +0700</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>BGN mewajibkan semua Satuan Pelayanan Pemenuhan Gizi (SPPG) atau dapur program Makan Bergizi Gratis (MBG) memiliki Sertifikat Laik Higiene Sanitasi (SLHS)</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606129/dapur-mbg-wajib-urus-slhs-paling-lambat-10-agustus-atau-tutup-permanen</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/27/32-ribu-pegawai-inti-mbg-bakal-diangkat-jadi-asn-pppk-1769488598601_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Fundamental Solid, Ekonomi Indonesia Triwulan II-2026 Tumbuh 5,29%</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:55:50 +0700</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Ekonomi Indonesia tumbuh 5,29% pada triwulan 2-2026, didorong konsumsi rumah tangga dan industri pengolahan. Fundamental ekonomi tetap solid.</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606079/fundamental-solid-ekonomi-indonesia-triwulan-ii-2026-tumbuh-5-29</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/05/kepala-bps-amalia-adininggar-widyasanti-1777954089390.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Satu Keluarga Keracunan MBG, Kepala BGN Ungkap Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:45:21 +0700</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN), Sudaryono mengungkap kasus keracunan Makan Begizi Gratis (MBG) yang menimpa satu keluarga.</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606069/satu-keluarga-keracunan-mbg-kepala-bgn-ungkap-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/tancap-gas-kepala-bgn-sudaryono-pecat-261-pegawai-bermasalah-1785138053252_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Beberapa Pabrik China Bakal Pindah ke Madura</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:09:33 +0700</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Beberapa pabrik asal China berencana direlokasi ke Kawasan Industri Madura di Bangkalan, Jawa Timur.</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/industri/d-8606022/beberapa-pabrik-china-bakal-pindah-ke-madura</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/07/31/ilustrasi-wanita-bekerja-di-pabrik_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Gaya Cristiano Ronaldo Jadi Pemilik Klub Spanyol</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:00:30 +0700</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Ronaldo nonton laga uji coba Al Nassr kontra Almeria di Portugal. Ronaldo menyaksikan dari tribune, dirinya adalah pemilik dari klub divisi dua Spanyol itu.</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/gila-bola/d-8605877/gaya-cristiano-ronaldo-jadi-pemilik-klub-spanyol</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/cristiano-ronaldo-almeria-1785914387259_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Bagaimana Nasib Mudryk di Chelsea? Ini Jawaban Xabi Alonso</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:45:35 +0700</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Mykhailo Mudryk sudah balik ke skuad Chelsea, ikut latihan di tur pramusim. Apa The Blues butuh tenaga sang winger, Xabi Alonso?</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8605875/bagaimana-nasib-mudryk-di-chelsea-ini-jawaban-xabi-alonso</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/12/25/myhailo-mudryk.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Audisi Umum PB Djarum 2026 Makassar Diikuti Peserta dari Berbagai Provinsi</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:35:30 +0700</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Audisi Umum PB Djarum 2026 berlangsung di Makassar, Sulawesi Selatan. Terakhir kali Kota Daeng disambangi terjadi satu dekade yang lalu.</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/raket/d-8605961/audisi-umum-pb-djarum-2026-makassar-diikuti-peserta-dari-berbagai-provinsi</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/bulutangkis-1785932121424_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Panitia soal Jadwal Padat Piala Presiden 2026</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:30:50 +0700</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Muhammad Robbani</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Panitia Piala Presiden 2026 menjelaskan alasan penerapan jadwal padat. Ditegaskan bahwa turnamen pramusim ini bukan kompetisi di bawah naungan FIFA.</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8606078/panitia-soal-jadwal-padat-piala-presiden-2026</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/06/ilustrasi-logo-piala-presiden-2026-1783328492093_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Yordania Merasa Sedang Diperas FIFA</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:15:15 +0700</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Presiden Asosiasi Sepakbola Yordania (JFA), Pangeran Ali bin Al Hussein, melontarkan kritik keras terhadap Presiden FIFA Gianni Infantino.</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8605871/yordania-merasa-sedang-diperas-fifa</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/16/fifa-logo-1784182664720_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Muaythai Naik Kelas, Menpora Puji Ketum PBMI</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:08:07 +0700</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Menteri Pemuda dan Olahraga (Menpora), Erick Thohir, memberikan apresiasi terhadap perkembangan Muaythai Indonesia.</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sport-lain/d-8606091/muaythai-naik-kelas-menpora-puji-ketum-pbmi</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/muaythai-1785938281839_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>2 Pemain yang Mesti Direkrut Arsenal untuk Naik Level</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:00:40 +0700</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Lucas Aditya</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Arsenal disarankan untuk merekrut salah satu dari dua pemain oleh eks pemain Tottenham Hotspur, Toby Alderweireld. Lini depan The Gunners harus ditingkatkan.</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8605873/2-pemain-yang-mesti-direkrut-arsenal-untuk-naik-level</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/22/soccer-worldcup-bra-hti-1782126575886_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Piala AFF 2026: Singapura Jamu Indonesia Jelang HUT Kemerdekaan</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:45:30 +0700</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Singapura menghadapi Indonesia pada laga penentuan Grup A Piala AFF 2026. The Lions menjamu Garuda dua hari jelang perayaan Hari Kemerdekaan.</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8605772/piala-aff-2026-singapura-jamu-indonesia-jelang-hut-kemerdekaan</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/12/26/egy-maulana-vikri-indonesia-vs-singapura_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Hasil Uji Coba Chelsea Vs Juventus: Bianconeri Menang 1-0</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:33:16 +0700</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Chelsea dan Juventus saling berhadapan di laga uji coba pramusim. Bianconeri yang berhasil menuntaskannya dengan kemenangan.</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8606054/hasil-uji-coba-chelsea-vs-juventus-bianconeri-menang-1-0</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/uji-coba-1785936703617_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Hasil Uji Coba: City Kalahkan K-League All Stars, Inter dan Milan Imbang</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:11:40 +0700</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Manchester City mengalahkan K-League All Stars di laga uji coba. Sementara itu, laga Inter Milan melawan AC Milan berakhir imbang.</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8606025/hasil-uji-coba-city-kalahkan-k-league-all-stars-inter-dan-milan-imbang</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/derby-milan-1785933385830_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Messi Donasi Rp1,7 Miliar untuk Korban Kebakaran Madrid</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:40:45 +0700</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Bayu Baskoro</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Aksi amal dilakukan Lionel Messi untuk wilayah pedesaan di Madrid yang jadi korban kebakaran. Legenda Barcelona ini mengirim donasi senilai Rp1,7 miliar.</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/gila-bola/d-8605770/messi-donasi-rp1-7-miliar-untuk-korban-kebakaran-madrid</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/tangis-messi-usai-argentina-gagal-pertahankan-gelar-juara-dunia-1784505521511_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>373,6 Hektare Kavling Laut Temuan Kementerian, BP Batam Sebut Sedang Lakukan Verifikasi</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:18:41 +0700</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>BP Batam tengah melakukan verifikasi terkait follow up pernyataan Kementerian ATR/BPN terkait kavling laut Batam mencapai 373,6 hektar.</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/05/221543678/3736-hektare-kavling-laut-temuan-kementerian-bp-batam-sebut-sedang-lakukan</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/zsbZJjf5cAtpRGhEEOWHKtmCLzs=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a730bb161773.jpg</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Sidang Korupsi Sudewo: Warga Pati Rela Berutang dan Habiskan Tabungan demi Mahar Perangkat Desa Rp 165 Juta</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:18:42 +0700</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Dia mengaku menjual perhiasan istrinya dan meminjam uang dari keluarga demi memenuhi permintaan uang Rp 165 juta untuk mengikuti seleksi perangkat.</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/05/213526378/sidang-korupsi-sudewo-warga-pati-rela-berutang-dan-habiskan-tabungan-demi</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/cKEvsm_2SpHUz6vBVfJKTS1KEcI=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a72e5cdb8810.jpg</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Terungkap Permintaan 'Aneh' Jared Leto Selama Syuting Film Tron: Ares</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:18:43 +0700</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Kebiasaan aneh Jared Leto saat syuting diungkap usai film dokumenternya jadi sorotan</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>https://entertainment.kompas.com/read/2026/08/05/210116766/terungkap-permintaan-aneh-jared-leto-selama-syuting-film-tron-ares</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/-brkW1MOHbYoZL3GlXnbAAHHkVA=/0x0:800x533/1200x675/filters:watermark(data/photo/2026/01/30/697c81706c5a3.png,0,-0,1)/data/photo/2017/10/04/3868250227.jpg</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I457"/>
+  <autoFilter ref="A1:I559"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-05 17:27 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-05.xlsx
+++ b/data/berita_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$559</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$605</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I559"/>
+  <dimension ref="A1:I605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -26707,8 +26707,2170 @@
         </is>
       </c>
     </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Purbaya: Kemenkeu ambil alih kepemilikan 60 persen saham di Whoosh</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:52:43 +0700</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan Kementerian Keuangan (Kemenkeu) akan mengambil alih kepemilikan 60 ...</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681728/purbaya-kemenkeu-ambil-alih-kepemilikan-60-persen-saham-di-whoosh</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000716076.jpg</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>KAI hentikan perjalanan kereta api karena gempa magintudo 5.3</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:52:17 +0700</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) Daerah Operasi 2 Bandung, Jawa Barat, menghentikan perjalanan Kereta Api Siliwangi ...</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681725/kai-hentikan-perjalanan-kereta-api-karena-gempa-magintudo-53</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/cek-kereta.jpg</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Kejari Kabupaten Madiun musnahkan barang bukti 21 perkara pidana</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:49:47 +0700</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Kejaksaan Negeri (Kejari) Kabupaten Madiun, Jawa Timur memusnahkan barang bukti dari 21 perkara pidana yang telah ...</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681721/kejari-kabupaten-madiun-musnahkan-barang-bukti-21-perkara-pidana</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/kajari-mdn.jpg</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Menhut tegaskan perdagangan karbon tak komersialisasi taman nasional</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:49:43 +0700</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Kehutanan Raja Juli Antoni di Jakarta, Rabu (5/8), menegaskan perdagangan karbon yang melibatkan hutan ...</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681715/menhut-tegaskan-perdagangan-karbon-tak-komersialisasi-taman-nasional</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENHUT-TEGASKAN-PERDAGANGAN-KARBON-TAK-KOMERSIALISASI-TAMAN-NASIONAL.jpg</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>CDC sebut Infeksi diare "eksplosif" merebak di 47 negara bagian AS</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:48:05 +0700</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Infeksi Siklosporiasis yang dapat menyebabkan diare "eksplosif" telah dilaporkan di 47 dari 50 negara bagian ...</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681719/cdc-sebut-infeksi-diare-eksplosif-merebak-di-47-negara-bagian-as</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/AmerikaSerikatBenderaPixabay.jpg</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>IPR: Masyarakat jangan terpancing soal konten hoaks aksi demonstrasi</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Direktur Indonesia Political Review (IPR) Iwan Setiawan mengajak masyarakat untuk tidak mudah terpancing oleh konten ...</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681717/ipr-masyarakat-jangan-terpancing-soal-konten-hoaks-aksi-demonstrasi</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/17/WhatsApp-Image-2026-07-17-at-18.02.04.jpeg</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Jabar jaga program prioritas di tengah defisit APBD</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:35:39 +0700</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Jawa Barat bersama DPRD Jawa Barat menyiapkan skema pinjaman daerah hingga Rp3,4 triliun ...</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681713/jabar-jaga-program-prioritas-di-tengah-defisit-apbd</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/JABAR-JAGA-PROGRAM-PRIORITAS-DI-TENGAH-DEFISIT-APBD.jpg</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Empat awak terluka dalam serangan terhadap kapal di Laut Hitam</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:29:13 +0700</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>ANTARA - Sebuah kapal kargo milik perusahaan pelayaran Turki dilaporkan diserang drone saat berlayar di Laut Hitam, ...</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681415/empat-awak-terluka-dalam-serangan-terhadap-kapal-di-laut-hitam</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-195245.jpg</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Program sejuta vaksin HPV sasar ASN dan masyarakat di Sulteng</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:25:43 +0700</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>ANTARA - Program Nasional Sejuta Vaksin HPV di Palu, Sulawesi Tengah menyasar aparatur sipil negara (ASN) dan ...</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681697/program-sejuta-vaksin-hpv-sasar-asn-dan-masyarakat-di-sulteng</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PROGRAM-SEJUTA-VAKSIN-HPV-SASAR-ASN-DAN-MASYARAKAT-DI-SULTENG.jpg</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Hadiah juara 2, 3, dan 4 Piala Presiden 2026 naik Rp500 juta</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:19:53 +0700</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Ketua Steering Committee (SC) Piala Presiden 2026 Maruarar Sirait resmi menaikkan hadiah juara 2, 3 dan 4 sebesar Rp500 ...</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681709/hadiah-juara-2-3-dan-4-piala-presiden-2026-naik-rp500-juta</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG-20260805-WA0017_1.jpg</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Saba Fest 3 gali potensi seni anak sejak dini</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:17:54 +0700</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Kebudayaan Provinsi Sumatera Barat melalui unit pelaksana teknis daerah (UPTD) Taman Budaya ...</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681648/saba-fest-3-gali-potensi-seni-anak-sejak-dini</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_25_24_19.Still478.jpg</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>DJKA uji jembatan KA usai peningkatan jalur Jember–Kalisat</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:10:12 +0700</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>ANTARA - Direktorat Jenderal Perkeretaapian Kementerian Perhubungan melalui Balai Teknik Perkeretaapian Kelas I ...</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681667/djka-uji-jembatan-ka-usai-peningkatan-jalur-jember-kalisat</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_27_47_27.Still479.jpg</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Ditjenpas NTT semarakkan HUT RI untuk perkuat pembinaan warga binaan</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:07:45 +0700</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>ANTARA - Kantor Wilayah Direktorat Jenderal Pemasyarakatan Nusa Tenggara Timur menggelar rangkaian kegiatan HUT Ke-81 ...</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681653/ditjenpas-ntt-semarakkan-hut-ri-untuk-perkuat-pembinaan-warga-binaan</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_DITJENPAS-NTT-SEMARAKKAN-HUT-RI-UNTUK-PERKUAT-PEMBINAAN-WARGA-BINAAN.jpg</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>KSP pastikan kesiapan Sekolah Rakyat saat MPLS dimulai</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:05:47 +0700</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>ANTARA - Sebanyak 560 siswa mengikuti Masa Pengenalan Lingkungan Sekolah (MPLS) di Sekolah Rakyat Terintegrasi 4 ...</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681649/ksp-pastikan-kesiapan-sekolah-rakyat-saat-mpls-dimulai</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KSP-PASTIKAN-KESIAPAN-SEKOLAH-RAKYAT-SAAT-MPLS-DIMULAI.jpg</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Menhut: 13 taman nasional jadi proyek percontohan pendanaan inovatif</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:57:28 +0700</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Kehutanan  Raja Juli Antoni menyebut terdapat 13 taman nasional yang menjadi proyek percontohan ...</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681681/menhut-13-taman-nasional-jadi-proyek-percontohan-pendanaan-inovatif</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENHUT-13-TAMAN-NASIONAL-JADI-PROYEK-PERCONTOHAN-PENDANAAN-INOVATIF.jpg</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Hensa klarifikasi ke Ditjen Pajak buntut siniar undang Ferry Latuhihin</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:54:16 +0700</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Pengamat politik sekaligus pendiri Lembaga Survei KedaiKOPI Hendri Satrio (Hensa) memberikan klarifikasi perihal ...</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681705/hensa-klarifikasi-ke-ditjen-pajak-buntut-siniar-undang-ferry-latuhihin</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Zulkieflimansyah.jpg</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Italia dorong dialog soal Selat Hormuz terus berlanjut</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:52:20 +0700</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Menteri Luar Negeri (Menlu) Italia Antonio Tajani menekankan pentingnya dialog terkait Selat Hormuz dalam pembicaraan ...</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681701/italia-dorong-dialog-soal-selat-hormuz-terus-berlanjut</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/04/15/Menlu-Italia-Antonio-Tajani.jpg</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>MRT Jakarta kembangkan TOD untuk pertumbuhan ekonomi dan mobilitas perkotaan</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:51:46 +0700</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>PT MRT Jakarta terus mengembangkan kawasan berorientasi transit (Transit Oriented Development/TOD) ...</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681699/mrt-jakarta-kembangkan-tod-untuk-pertumbuhan-ekonomi-dan-mobilitas-perkotaan</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/22/Progres-pembangunan-MRT-Fase-2A-220726-fzn-9.jpg</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Brussels perpanjang status waspada kekeringan</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:46:48 +0700</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Otoritas di Brussels, Belgia, memperpanjang status waspada kekeringan level kuning menyusul terus menurunnya ...</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681695/brussels-perpanjang-status-waspada-kekeringan</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/thumbs_b_59fbf283e2be22faf1b2d05596159eff.jpg</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Manufaktur lampaui ekonomi, Menperin: Industrialisasi di jalur tepat</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:44:14 +0700</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Menteri Perindustrian (Menperin) Agus Gumiwang Kartasasmita menyatakan manufaktur triwulan II 2026 yang tumbuh 5,32 ...</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681693/manufaktur-lampaui-ekonomi-menperin-industrialisasi-di-jalur-tepat</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/3-1_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Purbaya: Babinsa-Bhabinkamtibmas tak dikerahkan untuk pemungutan pajak</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:41:48 +0700</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa menegaskan pemerintah tidak mengerahkan Bintara Pembina Desa (Babinsa) maupun dan ...</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681692/purbaya-babinsa-bhabinkamtibmas-tak-dikerahkan-untuk-pemungutan-pajak</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-15.09.52_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Timnas 3x3 putri fokus benahi ketahanan fisik menuju AG 2026</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:41:43 +0700</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Pelatih timnas bola basket 3x3 putri Indonesia Deny Sartika mengatakan para pemainnya akan fokus membenahi ketahanan ...</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681689/timnas-3x3-putri-fokus-benahi-ketahanan-fisik-menuju-ag-2026</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/20/1000455403.jpg</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>China berkomitmen bantu negara-negara Afrika untuk perangi Ebola</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:40:11 +0700</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Juru bicara Kementerian Luar Negeri China Lin Jian pada Selasa (4/8) mengatakan bahwa dengan wabah Ebola yang masih ...</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681685/china-berkomitmen-bantu-negara-negara-afrika-untuk-perangi-ebola</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000011_20260805_CBMFN0A001.jpeg</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Pria bersenjata ditangkap di Klub Golf Milik Trump</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:37:34 +0700</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Departemen Sheriff Wilayah Los Angeles mengatakan pada Selasa (4/8) bahwa mereka telah menyerahkan kasus seorang pria ...</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681683/pria-bersenjata-ditangkap-di-klub-golf-milik-trump</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000024_20260805_CBMFN0A001.jpeg</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Kemenko Perekonomian nilai KI sumber pertumbuhan ekonomi masa depan</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:36:17 +0700</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Kementerian Koordinator (Kemenko) Bidang Perekonomian menilai kekayaan intelektual (KI) akan menjadi salah satu sumber ...</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681677/kemenko-perekonomian-nilai-ki-sumber-pertumbuhan-ekonomi-masa-depan</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000471691.jpg</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Wamenkop: Koperasi mampu kirim tenaga kerja profesional keluar negeri</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:34:12 +0700</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Koperasi (Wamenkop) Farida Farichah mengatakan koperasi mampu berperan dalam menyiapkan dan mengirim ...</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681675/wamenkop-koperasi-mampu-kirim-tenaga-kerja-profesional-keluar-negeri</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-19.09.11.jpeg</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Satelit Lampung-1 diluncurkan, buah kerja sama Indonesia-China</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:33:31 +0700</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Perusahaan antariksa komersial China, STAR.VISION, berhasil meluncurkan satelit Oriental Smart Eye (OSE) ...</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681671/satelit-lampung-1-diluncurkan-buah-kerja-sama-indonesia-china</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/z_2.jpg</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>DLH Makassar ajak masyarakat olah sampah organik sistem komunal</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:33:14 +0700</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Lingkungan Hidup Kota Makassar mengajak masyarakat mengolah sampah organik melalui sistem komunal di ...</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681432/dlh-makassar-ajak-masyarakat-olah-sampah-organik-sistem-komunal</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-05-200329.jpg</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>China perketat kontrol ekspor "drone" ke AS</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:33:12 +0700</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>China mulai memperketat pengawasan ekspor pesawat nirawak (drone) dan barang dwiguna terkait ke Amerika ...</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681668/china-perketat-kontrol-ekspor-drone-ke-as</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/07/XxjpbeE000059_20260507_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>AS catat 10.000 lebih kasus infeksi siklosporiasis sejak Mei 2026</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:25:27 +0700</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Pusat Pengendalian dan Pencegahan Penyakit Amerika Serikat (CDC) mencatat lebih dari 10.000 kasus infeksi ...</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681663/as-catat-10000-lebih-kasus-infeksi-siklosporiasis-sejak-mei-2026</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/AmerikaSerikatBenderaPixabay.jpg</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Pengamat dorong ATPM perkuat strategi hadapi sensitivitas konsumen</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:24:58 +0700</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Pengamat Ekonomi Senior dari Perbanas, Josua Pardede menilai bahwa Agen Tunggal Pemegang Merek (ATPM) perlu ...</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5681660/pengamat-dorong-atpm-perkuat-strategi-hadapi-sensitivitas-konsumen</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/48fd4b05-978c-4c12-bcef-6adeace5984d.jpeg</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Chery resmi kenalkan Tiggo V di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:23:37 +0700</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>PT Chery Sales Indonesia (CSI) memperkenalkan mobil terbaru mereka Tiggo V pada ajang pameran otomotif ...</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5681657/chery-resmi-kenalkan-tiggo-v-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-22.01.24.jpeg</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Polisi bantu kernet yang ditinggal sopir di Pelabuhan Tanjung Priok</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:20:12 +0700</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Kepolisian membantu seorang kernet bernama Akid, warga Cirebon, Jawa Barat yang kebingungan karena ditinggal ...</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681645/polisi-bantu-kernet-yang-ditinggal-sopir-di-pelabuhan-tanjung-priok</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/WhatsApp-Image-2026-08-05-at-21.08.58.jpeg</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Otto: Kekayaan intelektual potensi harta RI yang mesti dioptimalkan</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:18:31 +0700</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Koordinator Bidang Hukum, HAM, Imigrasi, dan Pemasyarakatan Otto Hasibuan mengatakan kekayaan intelektual ...</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681643/otto-kekayaan-intelektual-potensi-harta-ri-yang-mesti-dioptimalkan</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000471688.jpg</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Kemenkeu ambil alih restrukturisasi utang dan pengelolaan kereta cepat</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:17:38 +0700</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>ANTARA -Proses penyelesaian restrukturisasi utang dan pengelolaan kereta cepat Jakarta-Bandung kini diambil alih oleh ...</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681633/kemenkeu-ambil-alih-restrukturisasi-utang-dan-pengelolaan-kereta-cepat</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_KEMENKEU-AMBIL-ALIH-RESTRUKTURISASI-UTANG-DAN-PENGELOLAAN-KERETA-CEPAT.jpg</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Pura-pura pesan makan, pria di Kebon Jeruk gasak hp penjaga warung</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:13:35 +0700</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Seorang pria mencuri handphone milik penjaga warung makan di Jalan Pahlawan, Kebon Jeruk, Jakarta Barat, dengan modus ...</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681639/pura-pura-pesan-makan-pria-di-kebonjeruk-gasak-hp-penjaga-warung</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/06/30/penurian-hape.jpg</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>PT MRT investasikan Rp300 miliar bangun pedestrian deck Dukuh Atas</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:08:06 +0700</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>PT MRT menginvestasikan anggaran sebesar Rp300 miliar lebih untuk membangun pedestrian deck Dukuh Atas yang akan ...</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681637/pt-mrt-investasikan-rp300-miliar-bangun-pedestrian-deck-dukuh-atas</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/202607311821-main.cropped_1785496880.jpg</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>KSAU dan CAF RAAF bermanuver gunakan pesawat tempur di Australia</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:07:29 +0700</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Kepala Staf TNI Angkatan Udara (KSAU) Marsekal TNI Mohamad Tonny Harjono bermanuver menggunakan pesawat tempur bersama ...</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681635/ksau-dan-caf-raaf-bermanuver-gunakan-pesawat-tempur-di-australia</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001559265.jpg</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Cuaca Cerah Dimanfaatkan Petani China untuk Olah Hasil Panen Cabai</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:00:49 +0700</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Grandyos Zafna</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Petani di Bozhou, China, memanfaatkan cuaca cerah musim panas untuk memanen, menjemur, dan menyiapkan cabai sebelum dipasarkan.</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8604880/cuaca-cerah-dimanfaatkan-petani-china-untuk-olah-hasil-panen-cabai</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/cuaca-cerah-dimanfaatkan-petani-china-untuk-olah-hasil-panen-cabai-1785898636641.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>BGN Bakal Bangun Dapur MBG di Wilayah Tinggi Stunting</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:27:45 +0700</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>BGN tengah memetakan wilayah dengan tingkat stunting tinggi dan tinggi sekali di Indonesia. Pemetaan dilakukan untuk menyediakan dapur Makan Bergizi Gratis.</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606180/bgn-bakal-bangun-dapur-mbg-di-wilayah-tinggi-stunting</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/22/usai-dilantik-sudaryono-langsung-pimpin-rapat-perdana-bersama-jajaran-bgn-1784718690795_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Ekonomi Kuartal II Tumbuh 5,29%, Purbaya Nilai Cukup Baik</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:15:48 +0700</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa buka suara merespons pertumbuhan ekonomi di kuartal II-2026.</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606174/ekonomi-kuartal-ii-tumbuh-5-29-purbaya-nilai-cukup-baik</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/toko-online-lega-pemerintah-tunda-pajak-final-05-persen-1785929270093_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Serapan Tenaga Kerja Tembus 1,45 Juta Orang di Tengah Badai PHK</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Jumlah serapan tenaga kerja sepanjang semester I 2026 tembus 1,45 juta orang.</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606145/serapan-tenaga-kerja-tembus-1-45-juta-orang-di-tengah-badai-phk</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/03/08/mengintip-pabrik-travo-karya-anak-bangsa-demi-kemudahan-akses-iistrik-6_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Muay Aerobik Nusantara Jadi Aset Intelektual PBMI</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:15:48 +0700</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Randy Prasatya</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Muay Aerobik Nusantara menjadi bagian dari aset intelektual Pengurus Besar Muaythai Indonesia (PBMI)</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sport-lain/d-8606128/muay-aerobik-nusantara-jadi-aset-intelektual-pbmi</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/muaythai-1785939576697_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Rashford Memilih Bertahan di MU?</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:00:50 +0700</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Marcus Rashford akan segera gabung latihan pramusim Manchester United. Pihak klub masih buka opsi penjualan tapi sang winger fokus bertahan dulu.</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8605880/rashford-memilih-bertahan-di-mu</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/18/marcus-rashford-1781749340756.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Salah Sudah Tiba di Turki, Disambut bak Raja</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:40:20 +0700</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Mohammad Resha Pratama</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Mohamed Salah sudah tiba di Turki untuk menuntaskan kepindahannya ke Trabzonspor. Raja Mesir benar-benar disambut meriah fans klub tersebut.</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8606183/salah-sudah-tiba-di-turki-disambut-bak-raja</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/mohamed-salah-1785943966122_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Real Madrid Panen Cuan dari Jualan Pemain La Fabrica</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:20:50 +0700</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Bayu Baskoro</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Real Madrid tak hanya aktif dalam pembelian, tapi juga penjualan pemain. Los Merengues berhasil memecahkan rekor cuan dari penjualan penggawa-penggawa muda.</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8605631/real-madrid-panen-cuan-dari-jualan-pemain-la-fabrica</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/10/gonzalo-garcia-1754822037320_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I559"/>
+  <autoFilter ref="A1:I605"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-05 19:21 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-05.xlsx
+++ b/data/berita_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$605</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$613</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I605"/>
+  <dimension ref="A1:I613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -28869,8 +28869,384 @@
         </is>
       </c>
     </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>2 Jenazah Pendaki Gunung Piramid Bondowoso Berhasil Dievakuasi</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:50:10 +0700</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Chuk Shatu W</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Tim SAR berhasil evakuasi jenazah Maliya Finda dan pemandunya dari Gunung Piramid Bondowoso setelah 13 jam.</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606215/2-jenazah-pendaki-gunung-piramid-bondowoso-berhasil-dievakuasi</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/pendaki-gunung-piramid-1785945003710_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Israel Gerebek Kamp Pengungsi Palestina di Tepi Barat, 20 Orang Ditangkap</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:29:51 +0700</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Pasukan Israel menggerebek kamp pengungsian Palestina di Tepi Barat, menangkap 20 orang. Operasi ini dianggap sebagai intimidasi terhadap warga Palestina.</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606213/israel-gerebek-kamp-pengungsi-palestina-di-tepi-barat-20-orang-ditangkap</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/palestinian-israel-conflict-1785944818381_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Polisi Bongkar Kasus Pabrik Miras Ilegal di Bogor, 1 Orang Ditangkap</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:29:29 +0700</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Muchamad Sholihin</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Polsek Cileungsi ungkap kasus miras ilegal di Sukaraja, amankan pelaku M dan ratusan botol miras siap edar. Pelaku meracik miras sendiri untuk dijual.</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606212/polisi-bongkar-kasus-pabrik-miras-ilegal-di-bogor-1-orang-ditangkap</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/polsek-cileungsi-membongkar-kasus-minuman-keras-miras-ilegal-yang-diracik-di-sebuah-rumah-di-sukaraja-kabupaten-bogor-jawa-bar-1785947251444_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Polisi Malaysia Identifikasi Pemasok Narkoba yang Dibawa Pilot ke RI</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:52:31 +0700</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Polisi Malaysia identifikasi terduga pemasok narkoba ekstasi yang dibawa kopilot Malaysia Airlines ke Soekarno-Hatta. Penyelidikan berlanjut.</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606191/polisi-malaysia-identifikasi-pemasok-narkoba-yang-dibawa-pilot-ke-ri</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/rekaman-cctv-menunjukkan-gerak-gerik-kopilot-malaysia-airlines-sebelum-ditangkap-di-soetta-dok-instagram-bea-cukai-1785729571468_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Malaysia Kerahkan Polisi Jaga Bandara Buntut Pilot Selundupkan Narkoba ke RI</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:51:59 +0700</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Pemerintah Malaysia akan kerahkan polisi untuk perkuat keamanan bandara setelah penangkapan pilot yang menyelundupkan narkoba di Indonesia.</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606189/malaysia-kerahkan-polisi-jaga-bandara-buntut-pilot-selundupkan-narkoba-ke-ri</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/04/01/masuk-fase-awal-endemi-covid-19-malaysia-buka-pintu-buat-turis-asing-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Mendagri Siapkan 3 Langkah Solusi Operasional Gaji Pegawai Pemda</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:19:12 +0700</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Hana Nushratu</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Karnavian mengumumkan tiga langkah untuk membantu daerah yang kesulitan membayar gaji pegawai, termasuk efisiensi anggaran dan insentif DAU.</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606176/mendagri-siapkan-3-langkah-solusi-operasional-gaji-pegawai-pemda</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/kemendagri-1785943042201.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>4 Fakta Kebakaran Gedung di Cikini hingga Orang Terjebak Kepulan Asap</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:15:12 +0700</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda gedung di Cikini, Jakarta Pusat. Berikut sejumlah fakta yang diketahui.</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606172/4-fakta-kebakaran-gedung-di-cikini-hingga-orang-terjebak-kepulan-asap</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/kebakaran-gedung-di-cikini-jakarta-pusat-jakpus-dok-tmc-polda-metro-jaya-1785920371696.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>44.121 Huntap Akan Dibangun untuk Penyintas Bencana Sumatera</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:13:26 +0700</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Alfi Kholisdinuka</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Satgas PRR percepat pembangunan 44.121 hunian tetap untuk penyintas bencana di Aceh, Sumut, dan Sumbar. Fokus pada kualitas dan keamanan hunian.</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606170/44-121-huntap-akan-dibangun-untuk-penyintas-bencana-sumatera</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/44121-huntap-akan-dibangun-untuk-penyintas-bencana-1785942678207.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I605"/>
+  <autoFilter ref="A1:I613"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 01:29 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-05.xlsx
+++ b/data/berita_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$613</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$615</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I613"/>
+  <dimension ref="A1:I615"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -29245,8 +29245,102 @@
         </is>
       </c>
     </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Pensiun Jadi Wasit, Anthony Taylor Langsung Dapat Kerjaan Baru di Turki</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:30:45 +0700</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Kris FW</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Dua pekan setelah pensiun sebagai wasit, Anthony Taylor langsung mendapat jabatan penting di Federasi Sepakbola Turki (TFF).</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8605675/pensiun-jadi-wasit-anthony-taylor-langsung-dapat-kerjaan-baru-di-turki</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/09/17/anthony-taylor_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Duh, FIFA Ditagih 'Utang' Kota-kota AS Tuan Rumah Piala Dunia 2026</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 11:40:30 +0700</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Bayu Baskoro</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>FIFA kabarnya menjanjikan dana bantuan jutaan dolar AS untuk kota-kota tuan rumah Piala Dunia 2026. Janji tersebut rupanya belum dipenuhi.</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8604977/duh-fifa-ditagih-utang-kota-kota-as-tuan-rumah-piala-dunia-2026</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/12/logo-piala-dunia-2026-1781218052585_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I613"/>
+  <autoFilter ref="A1:I615"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 10:28 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-05.xlsx
+++ b/data/berita_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$615</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$660</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I615"/>
+  <dimension ref="A1:I660"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -29339,8 +29339,2123 @@
         </is>
       </c>
     </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Update Gempa M5,3 Pangandaran, Guncangan Dilaporkan Terasa di Bandung</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 23:05:15 +0700</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Gempa bumi tektonik M5.3 mengguncang Pangandaran, Jawa Barat, pada 5 Agustus 2026. Tidak berpotensi tsunami.</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805225612-20-1389102/update-gempa-m53-pangandaran-guncangan-dilaporkan-terasa-di-bandung</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2018/07/07/6101e4a4-1ee2-47a5-9838-13986a0c8632_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Anggota DPRD Bekasi Didakwa Lakukan Pengeroyokan hingga Korban Luka</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:50:21 +0700</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Jaksa menuntut anggota DPRD Bekasi, Nyumarno, dan dua lainnya atas kekerasan yang menyebabkan luka pada korban.</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805203837-12-1389081/anggota-dprd-bekasi-didakwa-lakukan-pengeroyokan-hingga-korban-luka</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/06/21/ilustrasi-hukum_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Ombak Tak Bersahabat, Warga Pulau Bawean Carter Pesawat Demi Rujuk Ibu</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:44:41 +0700</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Pengusaha di Pulau Bawean mencarter pesawat Rp110 juta demi ibunya guna dirujuk ke Surabaya karena gelombang tinggi yang membuat pelayaran terkendala.</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805202433-20-1389075/ombak-tak-bersahabat-warga-pulau-bawean-carter-pesawat-demi-rujuk-ibu</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/01/17/ilustrasi-pesawat-atr-atr-72-1768644498968_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Polisi Diduga Bunuh Nenek di Deliserdang Usai Ditolak Pinjam Uang</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:38:16 +0700</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Bripda RF, anggota polisi, membunuh nenek 70 tahun setelah ditolak meminjam uang Rp50 juta. Polresta telah mengungkapnya dalam tempo 2x24 jam.</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805164846-12-1388971/polisi-diduga-bunuh-nenek-di-deliserdang-usai-ditolak-pinjam-uang</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/08/09/ilustrasi-anggota-polisi-berseragam-dinas-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Gempa M5,3 di Pangandaran Jabar, Tak Berpotensi Tsunami</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:35:18 +0700</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Gempa berkekuatan M 5,3 terjadi di laut, sekitar 79 km barat daya Pangandaran, Jabar. tidak berpotensi tsunami.</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805223406-20-1389100/gempa-m53-di-pangandaran-jabar-tak-berpotensi-tsunami</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/11/16/6b71c58c-8a52-45c7-9e56-a1feb8e24c6a_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>FOTO: Penampakan JPO Kembar Rasuna Said, Berdampingan Tak Menyambung</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:17:43 +0700</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Dua jembatan penyeberangan orang (JPO) yang berdampingan di Jalan HR Rasuna Said, Jakarta Selatan, masih belum terhubung. Pemprov DKI berwacana menyambungnya.</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805200610-22-1389062/foto-penampakan-jpo-kembar-rasuna-said-berdampingan-tak-menyambung</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/jpo-kembar-rasuna-said-akan-terhubung-warga-tak-perlu-memutar-1785932475132_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Polisi Duga Pelaku Mutilasi di Depok adalah Penyuka Sesama Jenis</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:10:17 +0700</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Kasus mutilasi di Depok terungkap. Pelaku, Saepul, diduga penyuka sesama jenis atau LGBT dan mengaku terpaksa membunuh korban.</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805170415-12-1388979/polisi-duga-pelaku-mutilasi-di-depok-adalah-penyuka-sesama-jenis</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/09/26/ilustrasi-pasangan-lgbt_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Pengadilan Tipikor Mataram Vonis Bebas Ketua Komisi IV DPRD NTB</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 22:02:36 +0700</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Pengadilan Tipikor Mataram memvonis bebas Ketua Komisi IV DPRD NTB, Hamdan Kasim, dalam kasus gratifikasi. Hakim memulihkan hak-hak terdakwa.</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805200949-12-1389069/pengadilan-tipikor-mataram-vonis-bebas-ketua-komisi-iv-dprd-ntb</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/12/23/8f78cb8a-ccf2-4125-aa3a-a789a6b42b35_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Pemda DIY Tetapkan Raperda Larangan Perdagangan Daging Anjing</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:45:28 +0700</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Pemda DIY menetapkan Raperda larangan perdagangan daging anjing untuk melindungi kesehatan masyarakat dan mencegah penularan penyakit zoonosis.</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805175025-20-1388998/pemda-diy-tetapkan-raperda-larangan-perdagangan-daging-anjing</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2015/10/01/7fbc2857-28a1-415e-91c7-a13402daa01b_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Menkes Terima Kepala BGN, Didampingi Ahli Gizi Beri Masukan soal MBG</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:25:39 +0700</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Menkes Budi Gunadi Sadikin dan Kepala BGN Sudaryono bahas perbaikan program makan bergizi gratis. Ahli gizi diundang untuk masukan terkait menu dan layanan.</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805204317-20-1389085/menkes-terima-kepala-bgn-didampingi-ahli-gizi-beri-masukan-soal-mbg</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/menkes-terima-kepala-bgn-beri-masukan-soal-mbg-1785937187590_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Rektor Unsrat Manado Dicopot, Kemendikti Tunjuk Rektor Unhas Jadi Plt</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:20:27 +0700</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Rektor Universitas Hasanuddin, Prof Jamaluddin Jompa, ditunjuk sebagai Plt Rektor Universitas Sam Ratulangi, menggantikan Prof Oktovian yang dicopot.</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805145334-20-1388916/rektor-unsrat-manado-dicopot-kemendikti-tunjuk-rektor-unhas-jadi-plt</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/01/12/ilustrasi-toga-sarjana_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Dua Helikopter Dikerahkan Padamkan Kebakaran Bromo 80 Hektare</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:18:31 +0700</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>BNPB akan terjunkan helikopter dan drone untuk padamkan kebakaran hutan di Gunung Bromo. Kebakaran meluas hingga 80 hektare, penanganan ditargetkan cepat.</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805205427-20-1389087/dua-helikopter-dikerahkan-padamkan-kebakaran-bromo-80-hektare</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kebakaran-kawasan-bromo-meluas-hingga-80-hektare-pemadaman-pakai-drone-1785937271086_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Menkes Tanggapi Pasien BPJS Meninggal yang Sempat Dicibir Dokter</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:11:00 +0700</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>CNNIndonesia/Dela</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Menkes merespons beredarnya komentar sejumlah tenaga medis dan tenaga kesehatan di media sosial yang dinilai kurang berempati terhadap pasien BPJS.</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805202742-24-1389077/menkes-tanggapi-pasien-bpjs-meninggal-yang-sempat-dicibir-dokter</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kemenkes-tanggapi-kasus-pasien-bpjs-yang-meninggal-1785938018395_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>KPK Sebut Ada Penyerahan Sin$14.000 dari Bupati Kuansing ke Raja Juli</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:02:26 +0700</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>KPK mengungkap dugaan penyerahan uang Bupati Kuansing, Suhardiman Amby senilai Sin$14.000 ke Menhut Raja Juli.</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805194749-12-1389060/kpk-sebut-ada-penyerahan-sin-14000-dari-bupati-kuansing-ke-raja-juli</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/08/15/juru-bicara-kpk-budi-prasetyo-1755260853896_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Menkes Usai Pasien BPJS Dicibir Dokter Meninggal: Hati Saya Sedih</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:49:29 +0700</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Menkes Budi Gunadi merasa sedih atas meninggalnya pasien BPJS tak lama setelah dicibir dokter di media sosial.</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805202557-20-1389076/menkes-usai-pasien-bpjs-dicibir-dokter-meninggal-hati-saya-sedih</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/06/09/raker-komisi-ix-dpr-dengan-menkes-1780988911618_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Kebakaran Kawasan Bromo Meluas hingga 80 Hektare</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:40:14 +0700</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Gunung Bromo meluas hingga 80 hektare. Tim gabungan berupaya memadamkan api dengan drone water spray, akses wisata dibatasi demi keselamatan.</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805203717-20-1389080/kebakaran-kawasan-bromo-meluas-hingga-80-hektare</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/04/penutupan-sebagian-akses-wisata-bromo-1785849760126_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Kasus Dokter Cibir Pasien, UGM Dampingi Keluarga Pasien BPJS Meninggal</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:16:56 +0700</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>UGM memberikan pendampingan kepada keluarga pasien BPJS yang meninggal setelah komentar tak berempati dari dokter PPDS Elda Putri.</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805194541-12-1389059/kasus-dokter-cibir-pasien-ugm-dampingi-keluarga-pasien-bpjs-meninggal</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/05/15/universitas-gadjah-mada-1747298809962_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>FOTO: Pertengahan 2026, Penduduk Indonesia Tembus 290 Juta Jiwa</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:15:09 +0700</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Ditjen Dukcapil Kemendagri mencatat jumlah penduduk Indonesia mencapai 290.125.073 jiwa pada Juni 2026 atau pertengahan tahun ini.</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805184852-22-1389028/foto-pertengahan-2026-penduduk-indonesia-tembus-290-juta-jiwa</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/mobilitas-wni-di-saat-indonesia-capai-290-juta-jiwa-1785926921946_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Keluarga Mengaku Temukan Lebam di Jasad Mantan Istri Polisi Medan</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:06:27 +0700</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Kematian L (30) di Medan diduga bunuh diri, namun keluarga curiga. Mereka temukan luka lebam dan cekikan, menolak keterangan polisi.</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805192853-12-1389053/keluarga-mengaku-temukan-lebam-di-jasad-mantan-istri-polisi-medan</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/03/istri-polisi-diduga-bunuh-diri-pakai-senpi-di-medan-1785735979615_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>KPK Ungkap Pejabat Kemenhut Terima Sin$12.500 dari Bupati Kuansing</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:00:29 +0700</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>KPK mengungkap dugaan suap Bupati Kuansing, Suhardiman Amby, dengan pemberian uang Sin$12.500 terkait pelepasan kawasan hutan. Penyidikan berlanjut.</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805183600-12-1389027/kpk-ungkap-pejabat-kemenhut-terima-sin-12500-dari-bupati-kuansing</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/01/kpk-menetapkan-bupati-kuantan-singingi-kuansing-periode-2025-2030-suhardiman-amby-dan-sekretaris-daerah-zulkarnain-sebagai-ter-1782896232826_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Kebakaran di Gedung Cikini Diduga Berasal dari Lantai 3</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:43:16 +0700</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Kebakaran di gedung Ruko Central, Cikini, Jakarta Pusat, diduga berasal dari lantai 3. 22 mobil pemadam dikerahkan, tidak ada korban jiwa.</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805191219-20-1389047/kebakaran-di-gedung-cikini-diduga-berasal-dari-lantai-3</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kebakaran-proyek-ruko-di-cikini-1785929084828_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>FOTO: Kebakaran Proyek Ruko Lima Lantai di Cikini</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:22:50 +0700</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda proyek pembangunan ruko lima lantai di kawasan Central Cikini, Jalan Cikini Raya, Menteng, Jakarta Pusat, Rabu (5/8) sore.</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805182542-22-1389016/foto-kebakaran-proyek-ruko-lima-lantai-di-cikini</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kebakaran-proyek-ruko-di-cikini-1785928654250_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>UGM Investigasi Kasus Dokter PPDS Cibir Pasien BPJS</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:46:19 +0700</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>UGM menyelidiki dugaan komentar nirempati dokter PPDS Elda Putri terhadap pasien BPJS. Fakultas menyebut pentingnya etika dan empati dalam pelayanan kesehatan.</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805182548-20-1389014/ugm-investigasi-kasus-dokter-ppds-cibir-pasien-bpjs</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/05/15/universitas-gadjah-mada-1747298810268_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap Pria di Medan Produksi dan Jual Konten Gay Rp50 Ribu</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:20:14 +0700</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Polisi Medan menangkap BI alias Zilla, pria yang memproduksi dan menjual konten pornografi gay di aplikasi MiChat seharga Rp50.000.</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805175039-12-1388999/polisi-tangkap-pria-di-medan-produksi-dan-jual-konten-gay-rp50-ribu</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2015/07/24/0676200f-0af8-4c87-a754-bff6467e55d7_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Menko Polkam Buka Suara soal Fenomena Mal Pasang Pagar Tinggi</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:13:51 +0700</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Menko Polkam buka suara soal ramai pemasangan pagar tinggi di mall jelang isu demo Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805174510-12-1388997/menko-polkam-buka-suara-soal-fenomena-mal-pasang-pagar-tinggi</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kemenko-polkam-pastikan-situasi-nasional-aman-1785924470914_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Tito Imbau 16 K/L Segera Eksekusi Program Pascabencana Sumatra</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:52:20 +0700</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Karnavian mengumumkan 16 kementerian/lembaga telah menerima anggaran untuk rehabilitasi pascabencana Sumatra, Eksekusi program segera diperlukan.</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805174019-25-1388994/tito-imbau-16-k-l-segera-eksekusi-program-pascabencana-sumatra</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kemendagri-1785925591013_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Diduga Sebar Hoaks Demo, Perempuan Asal Ciamis Terancam 12 Tahun Bui</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:50:11 +0700</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Perempuan usia 45 tahun terancam 12 tahun penjara karena menyebarkan hoaks ajakan berdemo menjelang 17 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805150239-12-1388932/diduga-sebar-hoaks-demo-perempuan-asal-ciamis-terancam-12-tahun-bui</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/09/08/ilustrasi-tindakan-kriminal-5_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Eks Jampidsus Febrie Resmi Ajukan Praperadilan ke PN Jaksel</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:28:40 +0700</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Mantan Jaksa Agung Muda, Febrie Adriansyah, ajukan gugatan praperadilan terkait kasus TPPU. Pengacara uji proses hukum dan penetapan tersangka</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805172249-12-1388991/eks-jampidsus-febrie-resmi-ajukan-praperadilan-ke-pn-jaksel</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/25/febrie-adriansyah-ditahan-di-rutan-kpk-1784914679962_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Menteri PU Percepat SRT Kuantan Singingi, Patikan Siswa Aman dan Nyaman</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:26:13 +0700</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Menteri PU, Dody Hanggodo, dorong percepatan pembangunan SRT 1 Kuantan Singingi di Riau, dukung akses pendidikan berkualitas dan infrastruktur yang memadai.</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805165626-25-1388975/menteri-pu-percepat-srt-kuantan-singingi-patikan-siswa-aman-nyaman</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kementerian-pu-1785923006116_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>KemenPU Tuntaskan Pembangunan, 4 Sekolah Rakyat Sulsel Masuk MPLS</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:24:53 +0700</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Keempat Sekolah Rakyat Terintegrasi tersebut berada di Kabupaten Barru, Sidenreng Rappang (Sidrap), Tana Toraja, dan Bone, yang kini mulai melayani 1.508 siswa</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805170652-25-1388981/kemenpu-tuntaskan-pembangunan-4-sekolah-rakyat-sulsel-masuk-mpls</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kementerian-pu-1785923220363_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>KPK Sita Sin$8.500 Usai Geledah Kantor Imigrasi Jaksel-Jakpus</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:22:00 +0700</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>KPK menyita barang bukti terkait dugaan pemerasan izin tinggal WNA di Jakarta. Delapan tersangka telah ditahan, termasuk mantan Wakil Menteri Imigrasi.</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805171052-12-1388983/kpk-sita-sin-8500-usai-geledah-kantor-imigrasi-jaksel-jakpus</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/04/12/ilustrasi-dolar-singapura_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Bakom Investigasi Makalah MBG Diajukan untuk Nobel Perdamaian</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:10:54 +0700</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Pemerintah RI menyelidiki makalah yang mengusulkan program Makan Bergizi Gratis (MBG) sebagai kandidat Nobel Perdamaian 2026, melibatkan Prabowo Subianto.</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805163645-20-1388967/bakom-investigasi-makalah-mbg-diajukan-untuk-nobel-perdamaian</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/28/kepala-bakom-ri-minta-publik-fokus-substansi-soal-londo-ireng-1785244644776_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Karyawan SPPG Kuningan Korbankan Diri Cegah Babi Hutan Seruduk Bocah</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:07:50 +0700</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Anas, relawan SPPG, berkorban menahan babi hutan agar tidak menyerang anak-anak. Ia mengalami luka akibat gigitan babi, berharap kejadian serupa tak terulang.</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805154655-20-1388950/karyawan-sppg-kuningan-korbankan-diri-cegah-babi-hutan-seruduk-bocah</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/09/06/acef15ca-b1af-4e27-941d-3bca09048df2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Gus Ipul Tekankan Tiga Prioritas Pengelolaan Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:05:57 +0700</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Mensos Saifullah Yusuf atau Gus Ipul mengingatkan seluruh kepala Sekolah Rakyat di Indonesia untuk memprioritaskan tiga hal penting dalam pengelolaan sekolah.</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805170056-20-1388977/gus-ipul-tekankan-tiga-prioritas-pengelolaan-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kementerian-sosial-1785924188518_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Mendagri Ungkap 79 Pemda Butuh Rp3,7 Triliun untuk Bayar Gaji Pegawai</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:55:13 +0700</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Karnavian ungkap kebutuhan dana Rp3,5 triliun untuk belanja pegawai di 79 daerah.</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805163552-20-1388966/mendagri-ungkap-79-pemda-butuh-rp37-triliun-untuk-bayar-gaji-pegawai</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/29/mendagri-tito-karnavian-1780053714883_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Pemkab Musi Banyuasin Usulkan Lahan Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:41:00 +0700</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial menerima usulan lahan pembangunan Sekolah Rakyat dari Pemerintah Kabupaten Musi Banyuasin.</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805163557-20-1388965/pemkab-musi-banyuasin-usulkan-lahan-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kementerian-sosial-1785922534771_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Kemenkes Buka Suara soal Kasus Dokter Cibir Pasien BPJS di Medsos</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:40:56 +0700</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Kemenkes menanggapi cibiran dokter terhadap pasien BPJS Kesehatan di media sosial.</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805163301-20-1388964/kemenkes-buka-suara-soal-kasus-dokter-cibir-pasien-bpjs-di-medsos</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/02/12/rscm-tetap-berikan-pelayanan-meski-polemik-bjps-pbi-1770892442987_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Gus Ipul: Program Sekolah Rakyat Butuh Kolaborasi</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:39:48 +0700</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Menteri Sosial Saifullah Yusuf atau Gus Ipul menegaskan bahwa Sekolah Rakyat merupakan tanggung jawab bersama seluruh Unit Kerja (UKE) di Kementerian Sosial.</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805163221-20-1388963/gus-ipul-program-sekolah-rakyat-butuh-kolaborasi</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kementerian-sosial-1785922534966_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Gedung di Cikini Jakpus Kebakaran, 22 Mobil Damkar Diterjunkan</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:26:07 +0700</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda gedung Ruko Central di Cikini, Jakarta Pusat, pada Rabu sore. 22 unit mobil damkar dikerahkan untuk memadamkan api.</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805161904-20-1388959/gedung-di-cikini-jakpus-kebakaran-22-mobil-damkar-diterjunkan</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2020/01/01/2ab612fd-1f1a-4633-829b-795f0b6f1a1d_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Remaja di Buleleng Tepergok Diduga Curi Ayam Aduan, Berakhir Mediasi</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:22:55 +0700</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Dua remaja 16 tahun ditangkap karena mencuri ayam aduan di Buleleng, Bali. Mereka menjalani mediasi dan berjanji tidak mengulangi perbuatan.</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805153610-12-1388946/remaja-di-buleleng-tepergok-diduga-curi-ayam-aduan-berakhir-mediasi</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2015/03/31/68e08937-1493-47f7-8907-c81a726b33dc_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Kapolri Pastikan Tindak Pelaku Penyebaran Hoaks Demo</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:47:38 +0700</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Sigit memastikan pelaku penyebar hoaks demo akan ditindak. Masyarakat diingatkan untuk menyebarkan informasi yang akurat dan sesuai fakta.</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805151848-12-1388934/kapolri-pastikan-tindak-pelaku-penyebaran-hoaks-demo</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kumpulkan-panglima-tni-kapolri-menko-polkam-pastikan-kondisi-aman-terkendali-1785913030308_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>DPRD Beri Alarm soal Krisis Guru di Jabar, Kekurangan 6 Ribu Pengajar</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:40:52 +0700</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>DPRD Jabar soroti krisis kekurangan 6.000 guru. DPRD menilai hal itu bisa mengancam kualitas pendidikan dan masa depan generasi.</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805145755-20-1388920/dprd-beri-alarm-soal-krisis-guru-di-jabar-kekurangan-6-ribu-pengajar</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2016/08/09/2529fc07-7384-4cc6-9243-aa5c086272b5_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Menko Polkam Tegaskan Demo Diperbolehkan: Yang Dilarang Aksi Anarkis</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:26:29 +0700</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Menko Polkam Djamari Chaniago mengizinkan aksi demonstrasi asalkan tertib. Ia menegaskan kritik masyarakat penting dan situasi di Indonesia aman.</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805150035-12-1388921/menko-polkam-tegaskan-demo-diperbolehkan-yang-dilarang-aksi-anarkis</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/kumpulkan-panglima-tni-kapolri-menko-polkam-pastikan-kondisi-aman-terkendali-1785913030381_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>2 Pendaki Gunung PIramid Bondowoso yang Sempat Hilang Ditemukan Tewas</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:24:08 +0700</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Dua pendaki di Gunung Piramid, Bondowoso, ditemukan meninggal. Proses evakuasi dilakukan oleh tim SAR setelah penyisiran di lokasi kejadian.</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805150034-20-1388933/2-pendaki-gunung-piramid-bondowoso-yang-sempat-hilang-ditemukan-tewas</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/08/tim-sar-gabungan-cari-puluhan-pendaki-yang-tersesat-saat-gunung-dokuno-erupsi-1778218263491_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Kapolri Respons Isu Surpres</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 14:59:08 +0700</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Kapolri Listyo Sigit Prabowo menyatakan pergantian pimpinan Polri adalah hak prerogatif Presiden.</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805140047-12-1388892/kapolri-respons-isu-surpres</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/23/bazar-kreasi-bhayangkari-nusantara-kbn-2026-1784772703536_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I615"/>
+  <autoFilter ref="A1:I660"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 04:29 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-05.xlsx
+++ b/data/berita_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$798</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$834</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I798"/>
+  <dimension ref="A1:I834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -37940,8 +37940,1700 @@
         </is>
       </c>
     </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Laba Pengelola RS Hermina (HEAL) Anlok 14%, Ini Alasannya</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:10:17 +0700</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>PT Medikaloka Hermina Tbk. (HEAL) mencatat penurunan laba bersih 14,08% di paruh pertama 2026 meski pendapatan tumbuh 6,51% menjadi Rp3,60 triliun.</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805171008-17-756877/laba-pengelola-rs-hermina--heal--anlok-14-ini-alasannya</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/10/11/presiden-joko-widodo-jokowi-meresmikan-rumah-sakit-hermina-di-nusantara-kalimantan-timur-jumat-11102024-ia-menyebut-rumah-saki-2_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Perkuat Peran Perbankan, BRI Dukung Kebijakan Penempatan Dana SAL</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 21:09:19 +0700</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>BRI menyambut positif kebijakan penempatan dana SAL pemerintah untuk stabilitas likuiditas. Fokus pada penyaluran kredit berkualitas, terutama untuk UMKM.</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805210257-17-756931/perkuat-peran-perbankan-bri-dukung-kebijakan-penempatan-dana-sal</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/bri-1785938937254_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Purbaya Beri Sinyal China Mau Garap KA Cepat Bandung-Surabaya</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 20:05:32 +0700</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengungkapkan ketertarikan China untuk proyek kereta cepat hingga Jawa Timur, didukung oleh Presiden Prabowo Subianto.</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805185106-17-756907/purbaya-beri-sinyal-china-mau-garap-ka-cepat-bandung-surabaya</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/09/16/kereta-cepat-whoosh-1758006445490_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>WIKA Kebut Proyek Tol Jakarta-Cikampek II Selatan, Progres 85,20%</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:13:58 +0700</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>PT Wijaya Karya (WIKA) percepat pembangunan Jalan Tol Jakarta-Cikampek II Selatan Paket 2A dengan progres 85,20% dan target selesai Kuartal I 2027.</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805190921-17-756919/wika-kebut-proyek-tol-jakarta-cikampek-ii-selatan-progres-8520</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/jalan-tol-jakarta-cikampek-ii-selatan-1785932015629_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Bos Danantara Bocorkan IPO Pegadaian, Pelindo hingga Injourney</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 19:12:34 +0700</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Sejumlah perusahaan pelat merah atau Badan Usaha Milik Negara (BUMN) akan didorong untuk menjadi perusahaan publik dalam waktu dekat.</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805191039-17-756920/bos-danantara-bocorkan-ipo-pegadaian-pelindo-hingga-injourney</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/31/kepala-bp-bumn-sekaligus-coo-danantara-indonesia-dony-oskaria-saat-ditemui-di-istana-merdeka-jakarta-jumat-3172026-1785502950718_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Bos Kopi FORE Kasih Bocoran Soal Dividen</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:20:41 +0700</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Fore Kopi Indonesia belum dapat membagikan dividen karena saldo laba ditahan negatif. Namun, perusahaan berkomitmen untuk membagikan dividen di masa depan.</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805170540-17-756872/bos-kopi-fore-kasih-bocoran-soal-dividen</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/01/08/fore-coffee-dok-gallery-fore-2_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Purbaya Tambah Suntikan SAL Rp 70 T di Himbara, BTN dan BSI Dapat Jatah</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 18:11:38 +0700</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Robertus Andrianto</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Menkeu Purbaya Yudhi Sadewa menambah Rp70 triliun dana SAL ke Himbara. Suntikan dana dilakukan bertahap, dengan BTN dan BSI masing-masing Rp10 triliun.</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805180938-17-756903/purbaya-tambah-suntikan-sal-rp-70-t-di-himbara-btn-bsi-dapat-jatah</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/purbaya-yudhi-sadewa-menteri-keuangan-nufransa-wira-sakti-plt-direktur-jenderal-perimbangan-keuangan-dan-ubaidillah-amin-staf--1785916718720_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Video: Ekonomi RI H1-2026 Tumbuh 5,45%, Termasuk Tertinggi di ASEAN</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:49:07 +0700</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Airlangga: PDB RI H1-2026 Tumbuh 5,45%,Termasuk Tinggi di ASEAN</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805173341-19-756880/video-ekonomi-ri-h1-2026-tumbuh-545-termasuk-tertinggi-di-asean</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/airlangga-pdb-ri-h1-2026-tumbuh-545termasuk-tinggi-di-asean-1785926720666_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Pakai Strategi Ini, OJK Dorong BPD Kembangkan UMKM</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:45:11 +0700</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>OJK dorong BPD untuk kembangkan akses kredit bagi UMKM. Fokus pada ekosistem dan pendekatan community bank untuk memberdayakan masyarakat lokal.</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805172626-17-756878/pakai-strategi-ini-ojk-dorong-bpd-kembangkan-umkm</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/tak-hanya-andalkan-pemda-ojk-mau-bpd-kreatif-kumpulkan-dpk-ajak-warga-menabung-1785913789909_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Video: 3 Progam Grup KUB Bank Jatim, Dongkrak Kredit dan Digitalisasi</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:44:45 +0700</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>3 Progam Andalan Grup KUB Bank Jatim Dongkrak Kredit dan Layanan Digital BPD</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805161841-19-756842/video-3-progam-grup-kub-bank-jatim-dongkrak-kredit-digitalisasi</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/3-progam-andalan-grup-kub-bank-jatim-dongkrak-kredit-layanan-digital-bpd-1785922817327_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Laba Tembus Rp1,11 T, MTEL Genjot Pertumbuhan Bisnis di Luar Menara</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:28:19 +0700</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Mitratel mencatat pertumbuhan laba dan pendapatan yang solid di Semester I 2026, memperkuat transformasi menjadi Next-Gen Tower Company.</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805172455-17-756876/laba-tembus-rp111-t-mtel-genjot-pertumbuhan-bisnis-di-luar-menara</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/04/20/infrastruktur-digital_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>BEI Tambah Saham HSC, Ini Daftar Lengkap 54 Emiten Terbaru</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:20:21 +0700</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Mentari Puspadini</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Bursa Efek Indonesia menambah 55 saham dengan High Shareholding Concentration (HSC). Saham dikuasai entitas terkonsentrasi, meningkatkan risiko bagi investor.</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805170021-17-756869/bei-tambah-saham-hsc-ini-daftar-lengkap-54-emiten-terbaru</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797018492_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Bos BPD Ungkap Peluang Sinergi dengan BPR dan BPRS</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:12:24 +0700</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Teti Purwanti</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Industri BPD menjajaki kerja sama dengan BPR dan BPRS untuk sinergi yang saling menguntungkan. Kerja sama ini diharapkan mendorong akses layanan ke pasar mikro</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805165905-17-756868/bos-bpd-ungkap-peluang-sinergi-dengan-bpr-dan-bprs</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/direktur-utama-bank-jakarta-agus-haryoto-widodo-saat-menyampaikan-pemaparan-dalam-acara-regional-bank-summit-2026-di-jakarta-r-1785916201784_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Video: Bos Bank Jakarta: Ekonomi RI Tumbuh Positif, BPD Ikut Bertumbuh</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 17:12:00 +0700</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia TV</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Bos Bank Jakarta: Ekonomi RI Tumbuh Positif, BPD Mampu Jaga Pertumbuhan Aset dan Laba</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805161851-19-756840/video-bos-bank-jakarta-ekonomi-ri-tumbuh-positif-bpd-ikut-bertumbuh</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/bos-bank-jakarta-ekonomi-ri-tumbuh-positif-bpd-mampu-jaga-pertumbuhan-aset-dan-laba-1785922735158_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Purbaya Tegaskan Kemenkeu Ambil Alih Seluruh Saham BUMN di Whoosh</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:51:53 +0700</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Menkeu Purbaya Yudhi Sadewa memastikan utang KCIC akan diambil alih pemerintah. Konsorsium tetap ada, dengan 60% saham Indonesia dan 40% China.</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805164803-17-756853/purbaya-tegaskan-kemenkeu-ambil-alih-seluruh-saham-bumn-di-whoosh</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/purbaya-yudhi-sadewa-menteri-keuangan-nufransa-wira-sakti-plt-direktur-jenderal-perimbangan-keuangan-dan-ubaidillah-amin-staf--1785916718720_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Video: Bos Bank Jatim "Pamer" Keberhasilan Sinergi BPD Lewat KUB</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:49:07 +0700</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Bos Bank Jatim Pamer Keberhasilan Sinergi BPD Lewat KUB, Daya Saing Naik</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805161840-19-756838/video-bos-bank-jatim-pamer-keberhasilan-sinergi-bpd-lewat-kub</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/bos-bank-jatim-pamer-keberhasilan-sinergi-bpd-lewat-kub-daya-saing-naik-1785922771960_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Banyak Sentimen Positif, IHSG Menguat 0,5% ke Level 6.351</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:48:08 +0700</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>IHSG menguat 0,50% pada 5 Agustus 2026, didorong sentimen positif domestik dan global. Pertumbuhan ekonomi Indonesia kuartal II-2026 tumbuh 5,29% yoy.</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805163947-17-756851/banyak-sentimen-positif-ihsg-menguat-05-ke-level-6351</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797019138_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Video: Bank Jakarta dan BanK Jatim Soal Peran BPD Jadi Community Bank</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:43:00 +0700</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>OJK Dorong Peran BPD Jadi Community Bank di Daerah, Bos Bank Jakarta dan Bank Jatim Buka Suara</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805161844-19-756844/video-bank-jakarta-bank-jatim-soal-peran-bpd-jadi-community-bank</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/ojk-dorong-peran-bpd-jadi-community-bank-di-daerah-bos-bank-jakarta-bank-jatim-buka-suara-1785922902717_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Mesin Bisnis BNI Ngebut! Simpanan Nasabah Naik Rp 200 Triliun Setahun</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 16:15:02 +0700</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>BNI (BBNI) mencatat pertumbuhan solid di semester I-2026, dengan DPK meningkat Rp200 triliun dalam satu tahun.</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805135845-17-756765/mesin-bisnis-bni-ngebut-simpanan-nasabah-naik-rp-200-triliun-setahun</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/06/19/gedung-bank-negara-indonesia-bni-5_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Bos Bank Jatim Ungkap Tiga Kunci Keberhasilan BPD</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:59:42 +0700</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>Direktur Utama Bank Jatim, Winardi Legowo, menjelaskan keberhasilan BPD ditentukan oleh modal, sistem, dan SDM. KUB jadi strategi untuk tingkatkan daya saing.</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805155517-17-756825/bos-bank-jatim-ungkap-tiga-kunci-keberhasilan-bpd</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/direktur-utama-bank-jatim-winardi-legowo-saat-menyampaikan-pemaparan-dalam-acara-regional-bank-summit-2026-di-jakarta-rabu-582-1785917762527_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Kimia Farma (KAEF) Catat Laba Rp10,3 Miliar di Semester I-2026</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:51:13 +0700</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>PT Kimia Farma mencatat laba Rp10,32 miliar di semester I-2026, berbalik dari rugi Rp95,01 miliar tahun lalu, didorong peningkatan penjualan dan laba bruto.</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805154920-17-756820/kimia-farma--kaef--catat-laba-rp103-miliar-di-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/08/kimia-farma-1767867311774_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Rupiah Ditutup Menguat 0,50%, Dolar AS Turun ke Rp17.925</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 15:05:16 +0700</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Nilai tukar rupiah berhasil bangkit dan ditutup menguat terhadap dolar Amerika Serikat (AS).</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805145040-17-756793/rupiah-ditutup-menguat-050-dolar-as-turun-ke-rp17925</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/08/petugas-menjunjukkan-uang-pecahan-dolar-amerika-serikat-as-dan-rupiah-di-dolar-asia-money-changer-jakarta-rabu-872026-1783496342241_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Kredit BNI Nyaris Rp 1.000 Triliun, Tumbuh 24,4% Semester 1 2026</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 14:55:09 +0700</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>BNI menyalurkan kredit Rp968,5 triliun hingga semester I-2026, tumbuh 24,4% yoy.</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805131538-17-756746/kredit-bni-nyaris-rp-1000-triliun-tumbuh-244-semester-1-2026</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/09/26/gedung-bni_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Emiten Nagita Slavina (VISI) Rugi di Semester I-2026, Ini Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 14:40:52 +0700</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Satu Visi Putra (VISI) mencatat rugi bersih Rp4,17 miliar di semester I-2026, meski laba kotor tumbuh. Neraca menyusut setelah divestasi aset Rp75 miliar.</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805143114-17-756786/emiten-nagita-slavina--visi--rugi-di-semester-i-2026-ini-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797018756_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Swipe Sekali, Rp23 M Melayang! Ini Sisi Gelap Startup Live Belanja</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 14:05:33 +0700</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>Aplikasi belanja live streaming Whatnot menarik perhatian karena dampak adiktifnya. Pengguna menghabiskan jutaan dolar, memicu kritik dan gugatan hukum.</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805135155-17-756760/swipe-sekali-rp23-m-melayang-ini-sisi-gelap-startup-live-belanja</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/06/14/ilustrasi-belanja-online-dok-pixabay_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Asing Net Sell Rp65,81 Miliar di Sesi I, Ini Daftar Sahamnya</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 13:40:54 +0700</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>IHSG menguat 0,69% di tengah sentimen positif dari domestik dan global. Investor asing mencatat aksi jual bersih, terutama pada saham TLKM dan TPIA.</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805133258-17-756752/asing-net-sell-rp6581-miliar-di-sesi-i-ini-daftar-sahamnya</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/08/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-gedung-bursa-efek-indonesia-bei-jakarta-senin-862026-cnbc-ind-1780893013780_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Ada Kabar Baik dari Domestik dan Global, IHSG Naik 0,69% ke 6.363</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 12:36:50 +0700</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>IHSG menguat 0,69% di tengah sentimen positif dari domestik dan global. Ekonomi Indonesia tumbuh 5,29%, mendorong optimisme pasar. Baca selengkapnya!</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805120636-17-756729/ada-kabar-baik-dari-domestik-global-ihsg-naik-069-ke-6363</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797019966_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Breaking News! BNI (BBNI) Cetak Laba Rp10,8 T di Semester I-2026</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 11:31:03 +0700</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Bank Negara Indonesia (BNI) mencatat laba bersih Rp10,8 triliun di semester I-2026, tumbuh 5,94% yoy. Pendapatan bunga dan kualitas kredit juga meningkat.</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805112750-17-756702/breaking-news-bni--bbni--cetak-laba-rp108-t-di-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/09/26/gedung-bni_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Ekonomi RI Tumbuh 5,29%, IHSG Langsung Menguat 0,62%</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 11:26:21 +0700</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Gelson Kurniawan</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>BPS mengumumkan pertumbuhan ekonomi Indonesia kuartal II-2026 mencapai 5,29%, lebih tinggi dari ekspektasi. IHSG menguat 0,62% pasca pengumuman.</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805110849-17-756689/ekonomi-ri-tumbuh-529-ihsg-langsung-menguat-062</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797019966_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Ekonomi RI Tumbuh 5,29% dan Nilai Tukar Rupiah Menguat ke Rp17.905/US$</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 11:21:02 +0700</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Rupiah Garuda semakin menguat terhadap dolar Amerika Serikat (AS) pasca BPS umumkan pertumbuhan ekonomi kuartal II-2026.</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805111238-17-756692/ekonomi-ri-tumbuh-529-nilai-tukar-rupiah-menguat-ke-rp17905-us-</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/08/petugas-menjunjukkan-uang-pecahan-dolar-amerika-serikat-as-dan-rupiah-di-dolar-asia-money-changer-jakarta-rabu-872026-1783496342395_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>OJK Wajibkan Pindar Lapor Transaksi dan Larang Jual Beli Data Nasabah</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 11:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>OJK memperkuat regulasi industri Pinjaman Daring (Pindar) melalui penerbitan Peraturan Otoritas Jasa Keuangan (POJK) Nomor 8 Tahun 2026.</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805104901-17-756678/ojk-wajibkan-pindar-lapor-transaksi-dan-larang-jual-beli-data-nasabah</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/ilustrasi-seseorang-melakukan-pinjaman-online-dok-freepik-1785901803783_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Video: Harapan Damai di Selat Hormuz, Harga Minyak Emas dan Emas Anjlok</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 11:09:09 +0700</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Harapan Damai di Selat Hormuz, Harga Minyak Emas dan Emas Anjlok</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805103958-19-756677/video-harapan-damai-di-selat-hormuz-harga-minyak-emas-emas-anjlok</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/harapan-damai-di-selat-hormuz-harga-minyak-emas-emas-anjlok-1785902842826_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Dikabarkan Mau Caplok Raksasa Tambang Australia, Bos BUMI Buka Suara</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 10:45:30 +0700</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Emiten Grup Bakrie dan Salim, PT Bumi Resources Tbk (BUMI) memberikan klarifikasi atas rencana perseroan mengakuisisi Loyal Metals Limited.</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805102950-17-756674/dikabarkan-mau-caplok-raksasa-tambang-australia-bos-bumi-buka-suara</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/12/23/dok-bumi-resources-1_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Rombak Manajemen, Ini Susunan Direksi Terbaru Bank UOB Indonesia</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 10:10:52 +0700</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>PT Bank UOB Indonesia melakukan perubahan susunan direksi setelah masa jabatan salah satu direkturnya berakhir.</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805095051-17-756664/rombak-manajemen-ini-susunan-direksi-terbaru-bank-uob-indonesia</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/10/04/gedung-uob-indonesia-dok-uob-indonesia_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Video: Jelang Rilis PDB, IHSG Menghijau dan Rupiah Menguat</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 10:07:54 +0700</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Jelang Rilis PDB, IHSG Dibuka Menghijau dan Rupiah Menguat ke Rp 17.960 per USD</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805094511-19-756656/video-jelang-rilis-pdb-ihsg-menghijau-dan-rupiah-menguat</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/jelang-rilis-pdb-ihsg-dibuka-menghijau-rupiah-menguat-ke-rp-17960-per-usd-1785899124183_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>BEI Gembok Saham MDIA dan WIKA, Ini Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 10:00:49 +0700</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Romys Binekasri</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>BEI menghentikan sementara perdagangan (suspensi) saham PT Intermedia Capital Tbk (MDIA) dan memperpanjang suspensi saham PT Wijaya Karya (Persero) Tbk (WIKA).</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805094649-17-756657/bei-gembok-saham-mdia-dan-wika-ini-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797018492_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I798"/>
+  <autoFilter ref="A1:I834"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>